<commit_message>
Updated Safari Zone Encounters to include region-based encounters
</commit_message>
<xml_diff>
--- a/all_generations_pokemon_families.xlsx
+++ b/all_generations_pokemon_families.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3c6863eb3d429a98/Documents/GitHub/pokefirered-expansion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="742" documentId="8_{3DE7B663-32D8-4B09-ACF8-07A7237E0E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48789260-441F-45EA-AFB1-B38B8688DF15}"/>
+  <xr:revisionPtr revIDLastSave="775" documentId="8_{3DE7B663-32D8-4B09-ACF8-07A7237E0E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3F82EE78-4464-48E5-931E-8410CA463C16}"/>
   <bookViews>
     <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{913F818F-7E2F-42B8-8FB9-B28A63806581}"/>
   </bookViews>
@@ -4485,9 +4485,9 @@
     <col min="1" max="1" width="11.90625" bestFit="1" customWidth="1"/>
     <col min="2" max="8" width="8.7265625" hidden="1" customWidth="1"/>
     <col min="9" max="9" width="8.7265625" customWidth="1"/>
-    <col min="10" max="11" width="13.6328125" hidden="1" customWidth="1"/>
+    <col min="10" max="11" width="13.6328125" customWidth="1"/>
     <col min="12" max="13" width="8.7265625" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="27.6328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="27.6328125" hidden="1" customWidth="1"/>
     <col min="15" max="15" width="25.36328125" hidden="1" customWidth="1"/>
     <col min="16" max="16" width="12.36328125" bestFit="1" customWidth="1"/>
   </cols>
@@ -4542,7 +4542,7 @@
         <v>1194</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>41</v>
       </c>
@@ -4592,7 +4592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>779</v>
       </c>
@@ -4742,7 +4742,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>79</v>
       </c>
@@ -4792,7 +4792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>114</v>
       </c>
@@ -4842,7 +4842,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>46</v>
       </c>
@@ -4892,7 +4892,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>84</v>
       </c>
@@ -4942,7 +4942,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>84</v>
       </c>
@@ -4992,7 +4992,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>573</v>
       </c>
@@ -5042,7 +5042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>136</v>
       </c>
@@ -5092,7 +5092,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>515</v>
       </c>
@@ -5292,7 +5292,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>735</v>
       </c>
@@ -5342,7 +5342,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>739</v>
       </c>
@@ -5392,7 +5392,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>1039</v>
       </c>
@@ -5892,7 +5892,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>1045</v>
       </c>
@@ -5942,7 +5942,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>55</v>
       </c>
@@ -5992,7 +5992,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>535</v>
       </c>
@@ -6042,7 +6042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>653</v>
       </c>
@@ -6092,7 +6092,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>657</v>
       </c>
@@ -6142,7 +6142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>771</v>
       </c>
@@ -6192,7 +6192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>101</v>
       </c>
@@ -6242,7 +6242,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>108</v>
       </c>
@@ -6292,7 +6292,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>527</v>
       </c>
@@ -6342,7 +6342,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>552</v>
       </c>
@@ -6442,7 +6442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>813</v>
       </c>
@@ -6492,7 +6492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>1090</v>
       </c>
@@ -6542,7 +6542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>1053</v>
       </c>
@@ -6592,7 +6592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>857</v>
       </c>
@@ -6642,7 +6642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>1131</v>
       </c>
@@ -6692,7 +6692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>782</v>
       </c>
@@ -6742,7 +6742,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>782</v>
       </c>
@@ -6792,7 +6792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>798</v>
       </c>
@@ -6842,7 +6842,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>519</v>
       </c>
@@ -7142,7 +7142,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>606</v>
       </c>
@@ -7192,7 +7192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>91</v>
       </c>
@@ -7242,7 +7242,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>91</v>
       </c>
@@ -7542,7 +7542,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>122</v>
       </c>
@@ -7592,7 +7592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>152</v>
       </c>
@@ -7692,7 +7692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>220</v>
       </c>
@@ -8242,7 +8242,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>230</v>
       </c>
@@ -8292,7 +8292,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>230</v>
       </c>
@@ -8392,7 +8392,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>430</v>
       </c>
@@ -8442,7 +8442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>486</v>
       </c>
@@ -8542,7 +8542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>581</v>
       </c>
@@ -8592,7 +8592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>705</v>
       </c>
@@ -8642,7 +8642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>739</v>
       </c>
@@ -8742,7 +8742,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>793</v>
       </c>
@@ -8792,7 +8792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>804</v>
       </c>
@@ -8842,7 +8842,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>804</v>
       </c>
@@ -8892,7 +8892,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>819</v>
       </c>
@@ -8942,7 +8942,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>841</v>
       </c>
@@ -8992,7 +8992,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>845</v>
       </c>
@@ -9042,7 +9042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>887</v>
       </c>
@@ -9092,7 +9092,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>917</v>
       </c>
@@ -9142,7 +9142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>942</v>
       </c>
@@ -9192,7 +9192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>946</v>
       </c>
@@ -9242,7 +9242,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>961</v>
       </c>
@@ -9292,7 +9292,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="97" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>961</v>
       </c>
@@ -9342,7 +9342,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="98" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>968</v>
       </c>
@@ -9392,7 +9392,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="99" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>992</v>
       </c>
@@ -9442,7 +9442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="100" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>1117</v>
       </c>
@@ -9492,7 +9492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="101" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>1125</v>
       </c>
@@ -9542,7 +9542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="102" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>1143</v>
       </c>
@@ -9592,7 +9592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="103" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>863</v>
       </c>
@@ -9642,7 +9642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="104" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>48</v>
       </c>
@@ -9692,7 +9692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="105" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>156</v>
       </c>
@@ -9742,7 +9742,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="106" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>179</v>
       </c>
@@ -9792,7 +9792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="107" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>214</v>
       </c>
@@ -9892,7 +9892,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="109" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>546</v>
       </c>
@@ -9942,7 +9942,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="110" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>875</v>
       </c>
@@ -10242,7 +10242,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="116" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>26</v>
       </c>
@@ -10292,7 +10292,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="117" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>502</v>
       </c>
@@ -10342,7 +10342,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="118" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>1027</v>
       </c>
@@ -10392,7 +10392,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="119" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>207</v>
       </c>
@@ -10442,7 +10442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="120" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>270</v>
       </c>
@@ -10492,7 +10492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="121" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>288</v>
       </c>
@@ -10542,7 +10542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="122" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>384</v>
       </c>
@@ -10592,7 +10592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="123" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>384</v>
       </c>
@@ -10642,7 +10642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="124" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>717</v>
       </c>
@@ -10692,7 +10692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="125" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>723</v>
       </c>
@@ -10942,7 +10942,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="130" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>897</v>
       </c>
@@ -11542,7 +11542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="142" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>245</v>
       </c>
@@ -11592,7 +11592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="143" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>245</v>
       </c>
@@ -11642,7 +11642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="144" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>15</v>
       </c>
@@ -11692,7 +11692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="145" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>496</v>
       </c>
@@ -11742,7 +11742,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="146" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>1021</v>
       </c>
@@ -11942,7 +11942,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="150" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>319</v>
       </c>
@@ -11992,7 +11992,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="151" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>319</v>
       </c>
@@ -12042,7 +12042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="152" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>319</v>
       </c>
@@ -12092,7 +12092,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="153" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>542</v>
       </c>
@@ -12142,7 +12142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="154" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>119</v>
       </c>
@@ -12192,7 +12192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="155" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>256</v>
       </c>
@@ -12242,7 +12242,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="156" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>313</v>
       </c>
@@ -12292,7 +12292,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="157" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>313</v>
       </c>
@@ -12342,7 +12342,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="158" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>432</v>
       </c>
@@ -12392,7 +12392,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="159" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>432</v>
       </c>
@@ -12442,7 +12442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="160" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>432</v>
       </c>
@@ -12492,7 +12492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="161" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>432</v>
       </c>
@@ -12542,7 +12542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="162" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>432</v>
       </c>
@@ -12992,7 +12992,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="171" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
         <v>432</v>
       </c>
@@ -13042,7 +13042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="172" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
         <v>432</v>
       </c>
@@ -13092,7 +13092,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="173" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>432</v>
       </c>
@@ -13192,7 +13192,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="175" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
         <v>432</v>
       </c>
@@ -13242,7 +13242,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="176" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
         <v>432</v>
       </c>
@@ -13292,7 +13292,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="177" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
         <v>299</v>
       </c>
@@ -13542,7 +13542,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="182" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
         <v>1113</v>
       </c>
@@ -13592,7 +13592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="183" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
         <v>307</v>
       </c>
@@ -13642,7 +13642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="184" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
         <v>307</v>
       </c>
@@ -13742,7 +13742,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="186" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
         <v>682</v>
       </c>
@@ -13792,7 +13792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="187" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
         <v>686</v>
       </c>
@@ -13942,7 +13942,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="190" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
         <v>835</v>
       </c>
@@ -13992,7 +13992,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="191" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
         <v>881</v>
       </c>
@@ -14092,7 +14092,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="193" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
         <v>1135</v>
       </c>
@@ -14142,7 +14142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="194" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
         <v>1139</v>
       </c>
@@ -14192,7 +14192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="195" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
         <v>1153</v>
       </c>
@@ -14292,7 +14292,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="197" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
         <v>893</v>
       </c>
@@ -14342,7 +14342,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="198" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A198" t="s">
         <v>310</v>
       </c>
@@ -14392,7 +14392,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="199" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A199" t="s">
         <v>310</v>
       </c>
@@ -14442,7 +14442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="200" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
         <v>342</v>
       </c>
@@ -14592,7 +14592,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="203" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A203" t="s">
         <v>342</v>
       </c>
@@ -14742,7 +14742,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="206" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A206" t="s">
         <v>890</v>
       </c>
@@ -14792,7 +14792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="207" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A207" t="s">
         <v>1042</v>
       </c>
@@ -14842,7 +14842,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="208" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A208" t="s">
         <v>347</v>
       </c>
@@ -15442,7 +15442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="220" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
         <v>1101</v>
       </c>
@@ -15492,7 +15492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="221" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A221" t="s">
         <v>59</v>
       </c>
@@ -15542,7 +15542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="222" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
         <v>189</v>
       </c>
@@ -15592,7 +15592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="223" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A223" t="s">
         <v>189</v>
       </c>
@@ -15642,7 +15642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="224" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A224" t="s">
         <v>1059</v>
       </c>
@@ -15692,7 +15692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="225" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
         <v>1063</v>
       </c>
@@ -15742,7 +15742,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="226" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
         <v>1105</v>
       </c>
@@ -15792,7 +15792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="227" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
         <v>463</v>
       </c>
@@ -15842,7 +15842,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="228" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
         <v>467</v>
       </c>
@@ -15892,7 +15892,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="229" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
         <v>921</v>
       </c>
@@ -15942,7 +15942,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="230" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
         <v>925</v>
       </c>
@@ -15992,7 +15992,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="231" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
         <v>403</v>
       </c>
@@ -16042,7 +16042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="232" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
         <v>812</v>
       </c>
@@ -16092,7 +16092,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="233" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
         <v>1056</v>
       </c>
@@ -16142,7 +16142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="234" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
         <v>104</v>
       </c>
@@ -16192,7 +16192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="235" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
         <v>111</v>
       </c>
@@ -16292,7 +16292,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="237" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A237" t="s">
         <v>410</v>
       </c>
@@ -16342,7 +16342,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="238" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A238" t="s">
         <v>549</v>
       </c>
@@ -16442,7 +16442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="240" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A240" t="s">
         <v>522</v>
       </c>
@@ -16492,7 +16492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="241" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A241" t="s">
         <v>816</v>
       </c>
@@ -16642,7 +16642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="244" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A244" t="s">
         <v>294</v>
       </c>
@@ -16692,7 +16692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="245" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A245" t="s">
         <v>121</v>
       </c>
@@ -16742,7 +16742,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="246" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A246" t="s">
         <v>223</v>
       </c>
@@ -16792,7 +16792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="247" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A247" t="s">
         <v>233</v>
       </c>
@@ -16842,7 +16842,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="248" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A248" t="s">
         <v>233</v>
       </c>
@@ -16892,7 +16892,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="249" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A249" t="s">
         <v>233</v>
       </c>
@@ -16942,7 +16942,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="250" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A250" t="s">
         <v>233</v>
       </c>
@@ -16992,7 +16992,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="251" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A251" t="s">
         <v>473</v>
       </c>
@@ -17042,7 +17042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="252" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A252" t="s">
         <v>455</v>
       </c>
@@ -17092,7 +17092,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="253" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A253" t="s">
         <v>210</v>
       </c>
@@ -17142,7 +17142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="254" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A254" t="s">
         <v>210</v>
       </c>
@@ -17192,7 +17192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="255" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A255" t="s">
         <v>656</v>
       </c>
@@ -17242,7 +17242,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="256" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A256" t="s">
         <v>860</v>
       </c>
@@ -17342,7 +17342,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="258" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A258" t="s">
         <v>22</v>
       </c>
@@ -17392,7 +17392,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="259" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A259" t="s">
         <v>30</v>
       </c>
@@ -17492,7 +17492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="261" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A261" t="s">
         <v>213</v>
       </c>
@@ -17542,7 +17542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="262" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A262" t="s">
         <v>217</v>
       </c>
@@ -17592,7 +17592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="263" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A263" t="s">
         <v>217</v>
       </c>
@@ -17642,7 +17642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="264" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A264" t="s">
         <v>291</v>
       </c>
@@ -17692,7 +17692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="265" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A265" t="s">
         <v>291</v>
       </c>
@@ -17742,7 +17742,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="266" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A266" t="s">
         <v>499</v>
       </c>
@@ -17792,7 +17792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="267" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A267" t="s">
         <v>505</v>
       </c>
@@ -17842,7 +17842,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="268" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A268" t="s">
         <v>505</v>
       </c>
@@ -17942,7 +17942,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="270" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A270" t="s">
         <v>588</v>
       </c>
@@ -17992,7 +17992,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="271" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A271" t="s">
         <v>720</v>
       </c>
@@ -18042,7 +18042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="272" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A272" t="s">
         <v>726</v>
       </c>
@@ -18242,7 +18242,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="276" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A276" t="s">
         <v>1024</v>
       </c>
@@ -18292,7 +18292,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="277" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
         <v>1030</v>
       </c>
@@ -18392,7 +18392,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="279" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A279" t="s">
         <v>708</v>
       </c>
@@ -18442,7 +18442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="280" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A280" t="s">
         <v>971</v>
       </c>
@@ -18492,7 +18492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="281" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A281" t="s">
         <v>1048</v>
       </c>
@@ -18542,7 +18542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="282" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A282" t="s">
         <v>1128</v>
       </c>
@@ -18642,7 +18642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="284" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A284" t="s">
         <v>489</v>
       </c>
@@ -18692,7 +18692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="285" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A285" t="s">
         <v>995</v>
       </c>
@@ -18742,7 +18742,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="286" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A286" t="s">
         <v>518</v>
       </c>
@@ -18792,7 +18792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="287" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A287" t="s">
         <v>538</v>
       </c>
@@ -18842,7 +18842,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="288" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A288" t="s">
         <v>833</v>
       </c>
@@ -18892,7 +18892,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="289" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A289" t="s">
         <v>618</v>
       </c>
@@ -19292,7 +19292,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="297" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A297" t="s">
         <v>618</v>
       </c>
@@ -19342,7 +19342,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="298" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A298" t="s">
         <v>637</v>
       </c>
@@ -19492,7 +19492,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="301" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A301" t="s">
         <v>637</v>
       </c>
@@ -19542,7 +19542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="302" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A302" t="s">
         <v>637</v>
       </c>
@@ -19592,7 +19592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="303" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A303" t="s">
         <v>637</v>
       </c>
@@ -19642,7 +19642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="304" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A304" t="s">
         <v>838</v>
       </c>
@@ -19692,7 +19692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="305" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A305" t="s">
         <v>362</v>
       </c>
@@ -19742,7 +19742,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="306" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A306" t="s">
         <v>432</v>
       </c>
@@ -19792,7 +19792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="307" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A307" t="s">
         <v>593</v>
       </c>
@@ -19992,7 +19992,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="311" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A311" t="s">
         <v>801</v>
       </c>
@@ -20042,7 +20042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="312" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A312" t="s">
         <v>95</v>
       </c>
@@ -20092,7 +20092,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="313" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A313" t="s">
         <v>95</v>
       </c>
@@ -20142,7 +20142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="314" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A314" t="s">
         <v>159</v>
       </c>
@@ -20392,7 +20392,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="319" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A319" t="s">
         <v>530</v>
       </c>
@@ -20442,7 +20442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="320" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A320" t="s">
         <v>660</v>
       </c>
@@ -20492,7 +20492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="321" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A321" t="s">
         <v>1093</v>
       </c>
@@ -20792,7 +20792,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="327" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A327" t="s">
         <v>1093</v>
       </c>
@@ -20842,7 +20842,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="328" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A328" t="s">
         <v>139</v>
       </c>
@@ -20892,7 +20892,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="329" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A329" t="s">
         <v>183</v>
       </c>
@@ -20942,7 +20942,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="330" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A330" t="s">
         <v>811</v>
       </c>
@@ -20992,7 +20992,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="331" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A331" t="s">
         <v>389</v>
       </c>
@@ -21042,7 +21042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="332" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A332" t="s">
         <v>389</v>
       </c>
@@ -21092,7 +21092,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="333" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A333" t="s">
         <v>742</v>
       </c>
@@ -21142,7 +21142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="334" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A334" t="s">
         <v>742</v>
       </c>
@@ -21442,7 +21442,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="340" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A340" t="s">
         <v>844</v>
       </c>
@@ -21492,7 +21492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="341" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A341" t="s">
         <v>905</v>
       </c>
@@ -21542,7 +21542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="342" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A342" t="s">
         <v>907</v>
       </c>
@@ -21592,7 +21592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="343" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A343" t="s">
         <v>953</v>
       </c>
@@ -21642,7 +21642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="344" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A344" t="s">
         <v>155</v>
       </c>
@@ -21992,7 +21992,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="351" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A351" t="s">
         <v>324</v>
       </c>
@@ -22042,7 +22042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="352" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A352" t="s">
         <v>324</v>
       </c>
@@ -22092,7 +22092,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="353" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A353" t="s">
         <v>273</v>
       </c>
@@ -22142,7 +22142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="354" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A354" t="s">
         <v>738</v>
       </c>
@@ -22192,7 +22192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="355" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A355" t="s">
         <v>884</v>
       </c>
@@ -22292,7 +22292,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="357" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A357" t="s">
         <v>587</v>
       </c>
@@ -22492,7 +22492,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="361" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A361" t="s">
         <v>601</v>
       </c>
@@ -22542,7 +22542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="362" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A362" t="s">
         <v>774</v>
       </c>
@@ -22592,7 +22592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="363" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A363" t="s">
         <v>848</v>
       </c>
@@ -22642,7 +22642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="364" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A364" t="s">
         <v>879</v>
       </c>
@@ -22692,7 +22692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="365" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A365" t="s">
         <v>945</v>
       </c>
@@ -22742,7 +22742,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="366" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A366" t="s">
         <v>949</v>
       </c>
@@ -22792,7 +22792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="367" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A367" t="s">
         <v>61</v>
       </c>
@@ -22842,7 +22842,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="368" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A368" t="s">
         <v>1116</v>
       </c>
@@ -22892,7 +22892,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="369" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A369" t="s">
         <v>259</v>
       </c>
@@ -22942,7 +22942,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="370" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A370" t="s">
         <v>259</v>
       </c>
@@ -23042,7 +23042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="372" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A372" t="s">
         <v>680</v>
       </c>
@@ -23142,7 +23142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="374" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A374" t="s">
         <v>1108</v>
       </c>
@@ -23242,7 +23242,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="376" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A376" t="s">
         <v>822</v>
       </c>
@@ -23292,7 +23292,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="377" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A377" t="s">
         <v>350</v>
       </c>
@@ -23342,7 +23342,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="378" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A378" t="s">
         <v>878</v>
       </c>
@@ -23392,7 +23392,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="379" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A379" t="s">
         <v>896</v>
       </c>
@@ -23442,7 +23442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="380" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A380" t="s">
         <v>1044</v>
       </c>
@@ -23492,7 +23492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="381" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A381" t="s">
         <v>1123</v>
       </c>
@@ -23542,7 +23542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="382" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="382" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A382" t="s">
         <v>346</v>
       </c>
@@ -23592,7 +23592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="383" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="383" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A383" t="s">
         <v>367</v>
       </c>
@@ -23642,7 +23642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="384" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="384" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A384" t="s">
         <v>406</v>
       </c>
@@ -23742,7 +23742,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="386" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="386" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A386" t="s">
         <v>697</v>
       </c>
@@ -24092,7 +24092,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="393" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="393" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A393" t="s">
         <v>797</v>
       </c>
@@ -24142,7 +24142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="394" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="394" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A394" t="s">
         <v>302</v>
       </c>
@@ -24192,7 +24192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="395" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="395" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A395" t="s">
         <v>413</v>
       </c>
@@ -24392,7 +24392,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="399" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="399" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A399" t="s">
         <v>466</v>
       </c>
@@ -24442,7 +24442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="400" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="400" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A400" t="s">
         <v>470</v>
       </c>
@@ -24492,7 +24492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="401" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="401" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A401" t="s">
         <v>596</v>
       </c>
@@ -24542,7 +24542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="402" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="402" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A402" t="s">
         <v>866</v>
       </c>
@@ -24592,7 +24592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="403" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="403" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A403" t="s">
         <v>924</v>
       </c>
@@ -24642,7 +24642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="404" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="404" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A404" t="s">
         <v>928</v>
       </c>
@@ -24692,7 +24692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="405" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="405" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A405" t="s">
         <v>1062</v>
       </c>
@@ -24742,7 +24742,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="406" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="406" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A406" t="s">
         <v>1066</v>
       </c>
@@ -24942,7 +24942,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="410" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="410" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A410" t="s">
         <v>1104</v>
       </c>
@@ -24992,7 +24992,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="411" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="411" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A411" t="s">
         <v>89</v>
       </c>
@@ -25042,7 +25042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="412" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="412" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A412" t="s">
         <v>89</v>
       </c>
@@ -25142,7 +25142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="414" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="414" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A414" t="s">
         <v>293</v>
       </c>
@@ -25192,7 +25192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="415" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="415" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A415" t="s">
         <v>392</v>
       </c>
@@ -25242,7 +25242,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="416" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="416" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A416" t="s">
         <v>392</v>
       </c>
@@ -25292,7 +25292,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="417" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="417" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A417" t="s">
         <v>397</v>
       </c>
@@ -25342,7 +25342,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="418" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="418" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A418" t="s">
         <v>398</v>
       </c>
@@ -25392,7 +25392,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="419" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="419" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A419" t="s">
         <v>545</v>
       </c>
@@ -25442,7 +25442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="420" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="420" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A420" t="s">
         <v>609</v>
       </c>
@@ -25492,7 +25492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="421" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="421" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A421" t="s">
         <v>635</v>
       </c>
@@ -25542,7 +25542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="422" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="422" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A422" t="s">
         <v>685</v>
       </c>
@@ -25592,7 +25592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="423" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="423" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A423" t="s">
         <v>689</v>
       </c>
@@ -26042,7 +26042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="432" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="432" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A432" t="s">
         <v>920</v>
       </c>
@@ -26092,7 +26092,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="433" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="433" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A433" t="s">
         <v>1120</v>
       </c>
@@ -26142,7 +26142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="434" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="434" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A434" t="s">
         <v>1142</v>
       </c>
@@ -26192,7 +26192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="435" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="435" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A435" t="s">
         <v>1146</v>
       </c>
@@ -26242,7 +26242,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="436" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="436" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A436" t="s">
         <v>1156</v>
       </c>
@@ -26292,7 +26292,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="437" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="437" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A437" t="s">
         <v>107</v>
       </c>
@@ -26542,7 +26542,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="442" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="442" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A442" t="s">
         <v>113</v>
       </c>
@@ -26592,7 +26592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="443" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="443" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A443" t="s">
         <v>126</v>
       </c>
@@ -26642,7 +26642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="444" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="444" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A444" t="s">
         <v>633</v>
       </c>
@@ -26692,7 +26692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="445" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="445" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A445" t="s">
         <v>862</v>
       </c>
@@ -26942,7 +26942,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="450" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="450" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A450" t="s">
         <v>235</v>
       </c>
@@ -26992,7 +26992,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="451" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="451" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A451" t="s">
         <v>235</v>
       </c>
@@ -27142,7 +27142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="454" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="454" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A454" t="s">
         <v>249</v>
       </c>
@@ -27192,7 +27192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="455" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="455" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A455" t="s">
         <v>250</v>
       </c>
@@ -27292,7 +27292,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="457" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="457" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A457" t="s">
         <v>298</v>
       </c>
@@ -27342,7 +27342,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="458" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="458" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A458" t="s">
         <v>641</v>
       </c>
@@ -27392,7 +27392,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="459" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="459" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A459" t="s">
         <v>644</v>
       </c>
@@ -27442,7 +27442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="460" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="460" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A460" t="s">
         <v>900</v>
       </c>
@@ -27492,7 +27492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="461" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="461" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A461" t="s">
         <v>966</v>
       </c>
@@ -27542,7 +27542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="462" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="462" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A462" t="s">
         <v>967</v>
       </c>
@@ -27942,7 +27942,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="470" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="470" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A470" t="s">
         <v>459</v>
       </c>
@@ -27992,7 +27992,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="471" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="471" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A471" t="s">
         <v>471</v>
       </c>
@@ -28042,7 +28042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="472" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="472" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A472" t="s">
         <v>592</v>
       </c>
@@ -28092,7 +28092,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="473" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="473" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A473" t="s">
         <v>787</v>
       </c>
@@ -28142,7 +28142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="474" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="474" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A474" t="s">
         <v>788</v>
       </c>
@@ -28192,7 +28192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="475" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="475" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A475" t="s">
         <v>225</v>
       </c>
@@ -28242,7 +28242,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="476" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="476" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A476" t="s">
         <v>317</v>
       </c>
@@ -28292,7 +28292,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="477" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="477" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A477" t="s">
         <v>317</v>
       </c>
@@ -28392,7 +28392,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="479" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="479" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A479" t="s">
         <v>391</v>
       </c>
@@ -28442,7 +28442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="480" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="480" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A480" t="s">
         <v>551</v>
       </c>
@@ -28742,7 +28742,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="486" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="486" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A486" t="s">
         <v>605</v>
       </c>
@@ -28792,7 +28792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="487" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="487" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A487" t="s">
         <v>746</v>
       </c>
@@ -28842,7 +28842,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="488" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="488" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A488" t="s">
         <v>818</v>
       </c>
@@ -28892,7 +28892,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="489" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="489" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A489" t="s">
         <v>892</v>
       </c>
@@ -28942,7 +28942,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="490" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="490" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A490" t="s">
         <v>1058</v>
       </c>
@@ -28992,7 +28992,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="491" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="491" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A491" t="s">
         <v>24</v>
       </c>
@@ -29192,7 +29192,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="495" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="495" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A495" t="s">
         <v>219</v>
       </c>
@@ -29342,7 +29342,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="498" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="498" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A498" t="s">
         <v>448</v>
       </c>
@@ -29392,7 +29392,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="499" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="499" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A499" t="s">
         <v>449</v>
       </c>
@@ -29442,7 +29442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="500" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="500" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A500" t="s">
         <v>450</v>
       </c>
@@ -29492,7 +29492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="501" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="501" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A501" t="s">
         <v>451</v>
       </c>
@@ -29542,7 +29542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="502" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="502" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A502" t="s">
         <v>452</v>
       </c>
@@ -29592,7 +29592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="503" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="503" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A503" t="s">
         <v>453</v>
       </c>
@@ -29642,7 +29642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="504" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="504" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A504" t="s">
         <v>501</v>
       </c>
@@ -29692,7 +29692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="505" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="505" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A505" t="s">
         <v>622</v>
       </c>
@@ -29992,7 +29992,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="511" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="511" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A511" t="s">
         <v>952</v>
       </c>
@@ -30042,7 +30042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="512" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="512" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A512" t="s">
         <v>1026</v>
       </c>
@@ -30092,7 +30092,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="513" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="513" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A513" t="s">
         <v>1134</v>
       </c>
@@ -30142,7 +30142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="514" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="514" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A514" t="s">
         <v>1138</v>
       </c>
@@ -30292,7 +30292,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="517" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="517" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A517" t="s">
         <v>662</v>
       </c>
@@ -30342,7 +30342,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="518" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="518" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A518" t="s">
         <v>722</v>
       </c>
@@ -30392,7 +30392,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="519" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="519" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A519" t="s">
         <v>728</v>
       </c>
@@ -30442,7 +30442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="520" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="520" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A520" t="s">
         <v>840</v>
       </c>
@@ -30492,7 +30492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="521" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="521" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A521" t="s">
         <v>973</v>
       </c>
@@ -30592,7 +30592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="523" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="523" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A523" t="s">
         <v>32</v>
       </c>
@@ -30642,7 +30642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="524" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="524" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A524" t="s">
         <v>508</v>
       </c>
@@ -30692,7 +30692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="525" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="525" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A525" t="s">
         <v>508</v>
       </c>
@@ -30742,7 +30742,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="526" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="526" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A526" t="s">
         <v>1032</v>
       </c>
@@ -30792,7 +30792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="527" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="527" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A527" t="s">
         <v>141</v>
       </c>
@@ -30842,7 +30842,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="528" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="528" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A528" t="s">
         <v>187</v>
       </c>
@@ -30892,7 +30892,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="529" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="529" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A529" t="s">
         <v>353</v>
       </c>
@@ -30942,7 +30942,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="530" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="530" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A530" t="s">
         <v>366</v>
       </c>
@@ -31042,7 +31042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="532" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="532" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A532" t="s">
         <v>462</v>
       </c>
@@ -31192,7 +31192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="535" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="535" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A535" t="s">
         <v>409</v>
       </c>
@@ -31242,7 +31242,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="536" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="536" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A536" t="s">
         <v>416</v>
       </c>
@@ -31292,7 +31292,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="537" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="537" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A537" t="s">
         <v>476</v>
       </c>
@@ -31342,7 +31342,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="538" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="538" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A538" t="s">
         <v>576</v>
       </c>
@@ -31442,7 +31442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="540" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="540" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A540" t="s">
         <v>263</v>
       </c>
@@ -31592,7 +31592,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="543" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="543" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A543" t="s">
         <v>541</v>
       </c>
@@ -31642,7 +31642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="544" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="544" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A544" t="s">
         <v>193</v>
       </c>
@@ -31692,7 +31692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="545" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="545" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A545" t="s">
         <v>193</v>
       </c>
@@ -31742,7 +31742,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="546" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="546" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A546" t="s">
         <v>477</v>
       </c>
@@ -31792,7 +31792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="547" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="547" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A547" t="s">
         <v>477</v>
       </c>
@@ -31842,7 +31842,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="548" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="548" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A548" t="s">
         <v>480</v>
       </c>
@@ -31892,7 +31892,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="549" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="549" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A549" t="s">
         <v>480</v>
       </c>
@@ -32542,7 +32542,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="562" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="562" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A562" t="s">
         <v>483</v>
       </c>
@@ -32592,7 +32592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="563" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="563" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A563" t="s">
         <v>483</v>
       </c>
@@ -32642,7 +32642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="564" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="564" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A564" t="s">
         <v>699</v>
       </c>
@@ -32692,7 +32692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="565" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="565" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A565" t="s">
         <v>701</v>
       </c>
@@ -32992,7 +32992,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="571" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="571" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A571" t="s">
         <v>998</v>
       </c>
@@ -33042,7 +33042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="572" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="572" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A572" t="s">
         <v>1000</v>
       </c>
@@ -33092,7 +33092,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="573" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="573" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A573" t="s">
         <v>1002</v>
       </c>
@@ -33142,7 +33142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="574" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="574" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A574" t="s">
         <v>1164</v>
       </c>
@@ -33292,7 +33292,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="577" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="577" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A577" t="s">
         <v>1166</v>
       </c>
@@ -33342,7 +33342,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="578" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="578" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A578" t="s">
         <v>1168</v>
       </c>
@@ -33392,7 +33392,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="579" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="579" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A579" t="s">
         <v>491</v>
       </c>
@@ -33442,7 +33442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="580" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="580" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A580" t="s">
         <v>494</v>
       </c>
@@ -33542,7 +33542,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="582" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="582" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A582" t="s">
         <v>710</v>
       </c>
@@ -33592,7 +33592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="583" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="583" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A583" t="s">
         <v>715</v>
       </c>
@@ -33642,7 +33642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="584" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="584" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A584" t="s">
         <v>997</v>
       </c>
@@ -33692,7 +33692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="585" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="585" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A585" t="s">
         <v>1004</v>
       </c>
@@ -33742,7 +33742,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="586" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="586" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A586" t="s">
         <v>1006</v>
       </c>
@@ -33792,7 +33792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="587" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="587" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A587" t="s">
         <v>1014</v>
       </c>
@@ -33842,7 +33842,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="588" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="588" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A588" t="s">
         <v>1016</v>
       </c>
@@ -33892,7 +33892,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="589" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="589" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A589" t="s">
         <v>1016</v>
       </c>
@@ -33942,7 +33942,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="590" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="590" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A590" t="s">
         <v>1016</v>
       </c>
@@ -33992,7 +33992,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="591" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="591" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A591" t="s">
         <v>1016</v>
       </c>
@@ -34042,7 +34042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="592" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="592" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A592" t="s">
         <v>1130</v>
       </c>
@@ -34092,7 +34092,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="593" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="593" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A593" t="s">
         <v>1176</v>
       </c>
@@ -34292,7 +34292,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="597" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="597" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A597" t="s">
         <v>1183</v>
       </c>
@@ -34692,7 +34692,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="605" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="605" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A605" t="s">
         <v>1189</v>
       </c>
@@ -34742,7 +34742,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="606" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="606" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A606" t="s">
         <v>1191</v>
       </c>
@@ -34792,7 +34792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="607" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="607" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A607" t="s">
         <v>1191</v>
       </c>
@@ -34842,7 +34842,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="608" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="608" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A608" t="s">
         <v>803</v>
       </c>
@@ -34942,7 +34942,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="610" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="610" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A610" t="s">
         <v>1010</v>
       </c>
@@ -34992,7 +34992,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="611" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="611" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A611" t="s">
         <v>1178</v>
       </c>
@@ -35042,7 +35042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="612" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="612" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A612" t="s">
         <v>492</v>
       </c>
@@ -35092,7 +35092,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="613" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="613" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A613" t="s">
         <v>711</v>
       </c>
@@ -35142,7 +35142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="614" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="614" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A614" t="s">
         <v>713</v>
       </c>
@@ -35192,7 +35192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="615" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="615" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A615" t="s">
         <v>1012</v>
       </c>
@@ -35242,7 +35242,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="616" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="616" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A616" t="s">
         <v>1170</v>
       </c>
@@ -35292,7 +35292,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="617" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="617" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A617" t="s">
         <v>1170</v>
       </c>
@@ -35442,7 +35442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="620" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="620" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A620" t="s">
         <v>1180</v>
       </c>
@@ -35492,7 +35492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="621" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="621" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A621" t="s">
         <v>1180</v>
       </c>
@@ -35544,6 +35544,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:P621" xr:uid="{6A7ECD2C-6F5B-4E4D-962E-4B55F2FEEDC6}">
+    <filterColumn colId="9">
+      <filters>
+        <filter val="TYPE_WATER"/>
+      </filters>
+    </filterColumn>
     <filterColumn colId="15">
       <filters>
         <filter val="Y"/>

</xml_diff>

<commit_message>
Update trainer parties through mt moon
</commit_message>
<xml_diff>
--- a/all_generations_pokemon_families.xlsx
+++ b/all_generations_pokemon_families.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3c6863eb3d429a98/Documents/GitHub/pokefirered-expansion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="889" documentId="8_{3DE7B663-32D8-4B09-ACF8-07A7237E0E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{60FDAA18-FFB2-44B4-9137-D01E1BBD1DDC}"/>
+  <xr:revisionPtr revIDLastSave="903" documentId="8_{3DE7B663-32D8-4B09-ACF8-07A7237E0E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C143B821-1A07-4C49-9FEA-1095ABF7CE86}"/>
   <bookViews>
     <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{913F818F-7E2F-42B8-8FB9-B28A63806581}"/>
   </bookViews>
@@ -5042,7 +5042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="12" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>136</v>
       </c>
@@ -5142,7 +5142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>49</v>
       </c>
@@ -5192,7 +5192,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>52</v>
       </c>
@@ -5242,7 +5242,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>54</v>
       </c>
@@ -5442,7 +5442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>62</v>
       </c>
@@ -5492,7 +5492,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>65</v>
       </c>
@@ -5542,7 +5542,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>62</v>
       </c>
@@ -5592,7 +5592,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>62</v>
       </c>
@@ -5642,7 +5642,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>65</v>
       </c>
@@ -5692,7 +5692,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>71</v>
       </c>
@@ -5742,7 +5742,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>74</v>
       </c>
@@ -5792,7 +5792,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>75</v>
       </c>
@@ -5842,7 +5842,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>78</v>
       </c>
@@ -6192,7 +6192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="35" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>101</v>
       </c>
@@ -6242,7 +6242,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="36" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>108</v>
       </c>
@@ -6892,7 +6892,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>122</v>
       </c>
@@ -6942,7 +6942,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>126</v>
       </c>
@@ -6992,7 +6992,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>130</v>
       </c>
@@ -7042,7 +7042,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>133</v>
       </c>
@@ -7092,7 +7092,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>135</v>
       </c>
@@ -7292,7 +7292,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>142</v>
       </c>
@@ -7342,7 +7342,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>145</v>
       </c>
@@ -7392,7 +7392,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>145</v>
       </c>
@@ -7442,7 +7442,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>150</v>
       </c>
@@ -7492,7 +7492,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>151</v>
       </c>
@@ -7742,7 +7742,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>160</v>
       </c>
@@ -7792,7 +7792,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>163</v>
       </c>
@@ -7842,7 +7842,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>160</v>
       </c>
@@ -7892,7 +7892,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>163</v>
       </c>
@@ -7942,7 +7942,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>166</v>
       </c>
@@ -7992,7 +7992,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>169</v>
       </c>
@@ -8042,7 +8042,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>166</v>
       </c>
@@ -8092,7 +8092,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>169</v>
       </c>
@@ -8142,7 +8142,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>166</v>
       </c>
@@ -8192,7 +8192,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>174</v>
       </c>
@@ -8542,7 +8542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="82" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>581</v>
       </c>
@@ -9542,7 +9542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="102" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>1143</v>
       </c>
@@ -9592,7 +9592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="103" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>863</v>
       </c>
@@ -9992,7 +9992,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="111" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>239</v>
       </c>
@@ -10042,7 +10042,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="112" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>242</v>
       </c>
@@ -10092,7 +10092,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="113" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>239</v>
       </c>
@@ -10142,7 +10142,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="114" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>242</v>
       </c>
@@ -10792,7 +10792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="127" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>264</v>
       </c>
@@ -10842,7 +10842,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="128" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>264</v>
       </c>
@@ -10892,7 +10892,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="129" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>269</v>
       </c>
@@ -11042,7 +11042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="132" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>274</v>
       </c>
@@ -11092,7 +11092,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="133" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>277</v>
       </c>
@@ -11142,7 +11142,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="134" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>278</v>
       </c>
@@ -11192,7 +11192,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="135" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>281</v>
       </c>
@@ -11242,7 +11242,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="136" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>278</v>
       </c>
@@ -11292,7 +11292,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="137" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>281</v>
       </c>
@@ -11842,7 +11842,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="148" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>303</v>
       </c>
@@ -11892,7 +11892,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="149" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>306</v>
       </c>
@@ -12592,7 +12592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="163" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
         <v>325</v>
       </c>
@@ -12642,7 +12642,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="164" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
         <v>325</v>
       </c>
@@ -12692,7 +12692,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="165" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>325</v>
       </c>
@@ -12742,7 +12742,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="166" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
         <v>333</v>
       </c>
@@ -12792,7 +12792,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="167" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
         <v>334</v>
       </c>
@@ -12842,7 +12842,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="168" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
         <v>335</v>
       </c>
@@ -12892,7 +12892,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="169" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
         <v>336</v>
       </c>
@@ -12942,7 +12942,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="170" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
         <v>341</v>
       </c>
@@ -13142,7 +13142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="174" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
         <v>346</v>
       </c>
@@ -13342,7 +13342,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="178" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
         <v>354</v>
       </c>
@@ -13392,7 +13392,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="179" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
         <v>354</v>
       </c>
@@ -13442,7 +13442,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="180" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
         <v>359</v>
       </c>
@@ -13492,7 +13492,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="181" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
         <v>361</v>
       </c>
@@ -13542,7 +13542,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="182" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
         <v>1113</v>
       </c>
@@ -13842,7 +13842,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="188" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
         <v>376</v>
       </c>
@@ -13892,7 +13892,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="189" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
         <v>379</v>
       </c>
@@ -14142,7 +14142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="194" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
         <v>1139</v>
       </c>
@@ -14442,7 +14442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="200" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
         <v>342</v>
       </c>
@@ -14492,7 +14492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="201" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
         <v>399</v>
       </c>
@@ -14542,7 +14542,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="202" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A202" t="s">
         <v>402</v>
       </c>
@@ -14592,7 +14592,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="203" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A203" t="s">
         <v>342</v>
       </c>
@@ -14892,7 +14892,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="209" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A209" t="s">
         <v>417</v>
       </c>
@@ -14942,7 +14942,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="210" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A210" t="s">
         <v>419</v>
       </c>
@@ -14992,7 +14992,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="211" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A211" t="s">
         <v>419</v>
       </c>
@@ -15042,7 +15042,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="212" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A212" t="s">
         <v>419</v>
       </c>
@@ -15092,7 +15092,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="213" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A213" t="s">
         <v>419</v>
       </c>
@@ -15142,7 +15142,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="214" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A214" t="s">
         <v>424</v>
       </c>
@@ -15192,7 +15192,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="215" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A215" t="s">
         <v>427</v>
       </c>
@@ -16142,7 +16142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="234" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
         <v>104</v>
       </c>
@@ -16192,7 +16192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="235" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
         <v>111</v>
       </c>
@@ -16242,7 +16242,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="236" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A236" t="s">
         <v>454</v>
       </c>
@@ -18092,7 +18092,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="273" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A273" t="s">
         <v>523</v>
       </c>
@@ -18142,7 +18142,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="274" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A274" t="s">
         <v>526</v>
       </c>
@@ -18942,7 +18942,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="290" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A290" t="s">
         <v>558</v>
       </c>
@@ -18992,7 +18992,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="291" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A291" t="s">
         <v>561</v>
       </c>
@@ -19042,7 +19042,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="292" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A292" t="s">
         <v>562</v>
       </c>
@@ -19092,7 +19092,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="293" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A293" t="s">
         <v>565</v>
       </c>
@@ -19142,7 +19142,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="294" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A294" t="s">
         <v>567</v>
       </c>
@@ -19192,7 +19192,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="295" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A295" t="s">
         <v>568</v>
       </c>
@@ -19242,7 +19242,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="296" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A296" t="s">
         <v>572</v>
       </c>
@@ -19392,7 +19392,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="299" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A299" t="s">
         <v>577</v>
       </c>
@@ -19442,7 +19442,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="300" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A300" t="s">
         <v>580</v>
       </c>
@@ -19892,7 +19892,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="309" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A309" t="s">
         <v>597</v>
       </c>
@@ -19942,7 +19942,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="310" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A310" t="s">
         <v>600</v>
       </c>
@@ -20192,7 +20192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="315" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A315" t="s">
         <v>610</v>
       </c>
@@ -20242,7 +20242,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="316" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A316" t="s">
         <v>610</v>
       </c>
@@ -20292,7 +20292,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="317" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A317" t="s">
         <v>617</v>
       </c>
@@ -20342,7 +20342,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="318" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A318" t="s">
         <v>617</v>
       </c>
@@ -20542,7 +20542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="322" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A322" t="s">
         <v>623</v>
       </c>
@@ -20592,7 +20592,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="323" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A323" t="s">
         <v>626</v>
       </c>
@@ -20642,7 +20642,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="324" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A324" t="s">
         <v>627</v>
       </c>
@@ -20692,7 +20692,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="325" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A325" t="s">
         <v>627</v>
       </c>
@@ -20742,7 +20742,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="326" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A326" t="s">
         <v>632</v>
       </c>
@@ -20842,7 +20842,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="328" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A328" t="s">
         <v>139</v>
       </c>
@@ -21192,7 +21192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="335" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A335" t="s">
         <v>645</v>
       </c>
@@ -21242,7 +21242,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="336" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A336" t="s">
         <v>648</v>
       </c>
@@ -21292,7 +21292,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="337" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A337" t="s">
         <v>648</v>
       </c>
@@ -21342,7 +21342,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="338" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A338" t="s">
         <v>652</v>
       </c>
@@ -21392,7 +21392,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="339" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A339" t="s">
         <v>652</v>
       </c>
@@ -21692,7 +21692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="345" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A345" t="s">
         <v>663</v>
       </c>
@@ -21742,7 +21742,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="346" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A346" t="s">
         <v>663</v>
       </c>
@@ -21792,7 +21792,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="347" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A347" t="s">
         <v>667</v>
       </c>
@@ -21842,7 +21842,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="348" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A348" t="s">
         <v>668</v>
       </c>
@@ -21892,7 +21892,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="349" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A349" t="s">
         <v>671</v>
       </c>
@@ -21942,7 +21942,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="350" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A350" t="s">
         <v>672</v>
       </c>
@@ -22292,7 +22292,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="357" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A357" t="s">
         <v>587</v>
       </c>
@@ -22342,7 +22342,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="358" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A358" t="s">
         <v>690</v>
       </c>
@@ -22392,7 +22392,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="359" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A359" t="s">
         <v>694</v>
       </c>
@@ -22442,7 +22442,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="360" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A360" t="s">
         <v>695</v>
       </c>
@@ -22842,7 +22842,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="368" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A368" t="s">
         <v>1116</v>
       </c>
@@ -23542,7 +23542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="382" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="382" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A382" t="s">
         <v>346</v>
       </c>
@@ -23792,7 +23792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="387" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="387" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A387" t="s">
         <v>747</v>
       </c>
@@ -23842,7 +23842,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="388" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="388" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A388" t="s">
         <v>747</v>
       </c>
@@ -23892,7 +23892,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="389" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="389" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A389" t="s">
         <v>753</v>
       </c>
@@ -23942,7 +23942,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="390" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="390" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A390" t="s">
         <v>755</v>
       </c>
@@ -23992,7 +23992,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="391" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="391" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A391" t="s">
         <v>756</v>
       </c>
@@ -24042,7 +24042,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="392" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="392" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A392" t="s">
         <v>758</v>
       </c>
@@ -24242,7 +24242,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="396" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="396" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A396" t="s">
         <v>765</v>
       </c>
@@ -24292,7 +24292,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="397" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="397" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A397" t="s">
         <v>768</v>
       </c>
@@ -24342,7 +24342,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="398" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="398" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A398" t="s">
         <v>770</v>
       </c>
@@ -24542,7 +24542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="402" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="402" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A402" t="s">
         <v>866</v>
       </c>
@@ -24842,7 +24842,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="408" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="408" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A408" t="s">
         <v>789</v>
       </c>
@@ -24892,7 +24892,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="409" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="409" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A409" t="s">
         <v>792</v>
       </c>
@@ -25642,7 +25642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="424" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="424" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A424" t="s">
         <v>823</v>
       </c>
@@ -25692,7 +25692,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="425" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="425" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A425" t="s">
         <v>823</v>
       </c>
@@ -25742,7 +25742,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="426" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="426" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A426" t="s">
         <v>826</v>
       </c>
@@ -25792,7 +25792,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="427" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="427" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A427" t="s">
         <v>827</v>
       </c>
@@ -25842,7 +25842,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="428" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="428" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A428" t="s">
         <v>830</v>
       </c>
@@ -25892,7 +25892,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="429" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="429" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A429" t="s">
         <v>831</v>
       </c>
@@ -26142,7 +26142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="434" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="434" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A434" t="s">
         <v>1142</v>
       </c>
@@ -26192,7 +26192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="435" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="435" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A435" t="s">
         <v>1146</v>
       </c>
@@ -26292,7 +26292,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="437" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="437" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A437" t="s">
         <v>107</v>
       </c>
@@ -26342,7 +26342,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="438" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="438" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A438" t="s">
         <v>849</v>
       </c>
@@ -26392,7 +26392,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="439" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="439" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A439" t="s">
         <v>851</v>
       </c>
@@ -26442,7 +26442,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="440" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="440" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A440" t="s">
         <v>853</v>
       </c>
@@ -26492,7 +26492,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="441" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="441" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A441" t="s">
         <v>855</v>
       </c>
@@ -26542,7 +26542,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="442" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="442" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A442" t="s">
         <v>113</v>
       </c>
@@ -26792,7 +26792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="447" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="447" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A447" t="s">
         <v>867</v>
       </c>
@@ -26842,7 +26842,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="448" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="448" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A448" t="s">
         <v>870</v>
       </c>
@@ -27142,7 +27142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="454" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="454" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A454" t="s">
         <v>249</v>
       </c>
@@ -27192,7 +27192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="455" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="455" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A455" t="s">
         <v>250</v>
       </c>
@@ -27242,7 +27242,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="456" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="456" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A456" t="s">
         <v>885</v>
       </c>
@@ -27642,7 +27642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="464" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="464" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A464" t="s">
         <v>901</v>
       </c>
@@ -27692,7 +27692,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="465" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="465" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A465" t="s">
         <v>903</v>
       </c>
@@ -27842,7 +27842,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="468" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="468" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A468" t="s">
         <v>909</v>
       </c>
@@ -27892,7 +27892,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="469" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="469" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A469" t="s">
         <v>912</v>
       </c>
@@ -28492,7 +28492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="481" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="481" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A481" t="s">
         <v>935</v>
       </c>
@@ -28542,7 +28542,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="482" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="482" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A482" t="s">
         <v>935</v>
       </c>
@@ -28592,7 +28592,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="483" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="483" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A483" t="s">
         <v>935</v>
       </c>
@@ -28642,7 +28642,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="484" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="484" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A484" t="s">
         <v>935</v>
       </c>
@@ -28692,7 +28692,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="485" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="485" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A485" t="s">
         <v>940</v>
       </c>
@@ -29042,7 +29042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="492" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="492" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A492" t="s">
         <v>955</v>
       </c>
@@ -29092,7 +29092,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="493" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="493" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A493" t="s">
         <v>958</v>
       </c>
@@ -29142,7 +29142,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="494" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="494" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A494" t="s">
         <v>959</v>
       </c>
@@ -29742,7 +29742,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="506" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="506" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A506" t="s">
         <v>982</v>
       </c>
@@ -29792,7 +29792,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="507" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="507" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A507" t="s">
         <v>984</v>
       </c>
@@ -29842,7 +29842,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="508" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="508" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A508" t="s">
         <v>986</v>
       </c>
@@ -29892,7 +29892,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="509" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="509" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A509" t="s">
         <v>989</v>
       </c>
@@ -29942,7 +29942,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="510" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="510" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A510" t="s">
         <v>991</v>
       </c>
@@ -30792,7 +30792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="527" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="527" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A527" t="s">
         <v>141</v>
       </c>
@@ -31492,7 +31492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="541" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="541" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A541" t="s">
         <v>1049</v>
       </c>
@@ -31542,7 +31542,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="542" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="542" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A542" t="s">
         <v>1052</v>
       </c>
@@ -31942,7 +31942,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="550" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="550" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A550" t="s">
         <v>1067</v>
       </c>
@@ -31992,7 +31992,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="551" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="551" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A551" t="s">
         <v>1067</v>
       </c>
@@ -32042,7 +32042,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="552" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="552" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A552" t="s">
         <v>1067</v>
       </c>
@@ -32092,7 +32092,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="553" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="553" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A553" t="s">
         <v>1067</v>
       </c>
@@ -32142,7 +32142,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="554" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="554" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A554" t="s">
         <v>1067</v>
       </c>
@@ -32192,7 +32192,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="555" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="555" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A555" t="s">
         <v>1067</v>
       </c>
@@ -32242,7 +32242,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="556" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="556" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A556" t="s">
         <v>1079</v>
       </c>
@@ -32292,7 +32292,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="557" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="557" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A557" t="s">
         <v>1079</v>
       </c>
@@ -32342,7 +32342,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="558" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="558" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A558" t="s">
         <v>1079</v>
       </c>
@@ -32392,7 +32392,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="559" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="559" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A559" t="s">
         <v>1080</v>
       </c>
@@ -32442,7 +32442,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="560" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="560" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A560" t="s">
         <v>1083</v>
       </c>
@@ -32492,7 +32492,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="561" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="561" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A561" t="s">
         <v>1084</v>
       </c>
@@ -32792,7 +32792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="567" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="567" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A567" t="s">
         <v>1095</v>
       </c>
@@ -32842,7 +32842,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="568" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="568" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A568" t="s">
         <v>1095</v>
       </c>
@@ -32892,7 +32892,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="569" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="569" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A569" t="s">
         <v>1100</v>
       </c>
@@ -32942,7 +32942,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="570" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="570" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A570" t="s">
         <v>1100</v>
       </c>
@@ -33192,7 +33192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="575" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="575" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A575" t="s">
         <v>1109</v>
       </c>
@@ -33242,7 +33242,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="576" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="576" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A576" t="s">
         <v>1112</v>
       </c>
@@ -33492,7 +33492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="581" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="581" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A581" t="s">
         <v>1121</v>
       </c>
@@ -34142,7 +34142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="594" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="594" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A594" t="s">
         <v>1147</v>
       </c>
@@ -34192,7 +34192,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="595" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="595" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A595" t="s">
         <v>1149</v>
       </c>
@@ -34242,7 +34242,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="596" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="596" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A596" t="s">
         <v>1152</v>
       </c>
@@ -34392,7 +34392,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="599" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="599" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A599" t="s">
         <v>1157</v>
       </c>
@@ -34442,7 +34442,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="600" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="600" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A600" t="s">
         <v>1157</v>
       </c>
@@ -34492,7 +34492,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="601" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="601" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A601" t="s">
         <v>1157</v>
       </c>
@@ -34542,7 +34542,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="602" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="602" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A602" t="s">
         <v>1157</v>
       </c>
@@ -34592,7 +34592,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="603" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="603" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A603" t="s">
         <v>1157</v>
       </c>
@@ -34642,7 +34642,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="604" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="604" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A604" t="s">
         <v>1157</v>
       </c>
@@ -35544,9 +35544,14 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:P621" xr:uid="{6A7ECD2C-6F5B-4E4D-962E-4B55F2FEEDC6}">
+    <filterColumn colId="9">
+      <filters>
+        <filter val="TYPE_POISON"/>
+      </filters>
+    </filterColumn>
     <filterColumn colId="15">
       <filters>
-        <filter val="N"/>
+        <filter val="Y"/>
       </filters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P621">

</xml_diff>

<commit_message>
Update to rival parties
</commit_message>
<xml_diff>
--- a/all_generations_pokemon_families.xlsx
+++ b/all_generations_pokemon_families.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3c6863eb3d429a98/Documents/GitHub/pokefirered-expansion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="903" documentId="8_{3DE7B663-32D8-4B09-ACF8-07A7237E0E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C143B821-1A07-4C49-9FEA-1095ABF7CE86}"/>
+  <xr:revisionPtr revIDLastSave="911" documentId="8_{3DE7B663-32D8-4B09-ACF8-07A7237E0E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C352AAC-F15E-4A9F-A033-83CC755FFAC0}"/>
   <bookViews>
     <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{913F818F-7E2F-42B8-8FB9-B28A63806581}"/>
   </bookViews>
@@ -5042,7 +5042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>136</v>
       </c>
@@ -6192,7 +6192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>101</v>
       </c>
@@ -6242,7 +6242,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>108</v>
       </c>
@@ -8542,7 +8542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>581</v>
       </c>
@@ -9142,7 +9142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="94" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>942</v>
       </c>
@@ -9192,7 +9192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="95" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>946</v>
       </c>
@@ -9542,7 +9542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="102" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>1143</v>
       </c>
@@ -9592,7 +9592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="103" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>863</v>
       </c>
@@ -10492,7 +10492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="121" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>288</v>
       </c>
@@ -13542,7 +13542,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="182" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
         <v>1113</v>
       </c>
@@ -14142,7 +14142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="194" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
         <v>1139</v>
       </c>
@@ -14442,7 +14442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="200" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
         <v>342</v>
       </c>
@@ -14592,7 +14592,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="203" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A203" t="s">
         <v>342</v>
       </c>
@@ -15442,7 +15442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="220" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
         <v>1101</v>
       </c>
@@ -16142,7 +16142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="234" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
         <v>104</v>
       </c>
@@ -16192,7 +16192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="235" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
         <v>111</v>
       </c>
@@ -17642,7 +17642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="264" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A264" t="s">
         <v>291</v>
       </c>
@@ -17692,7 +17692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="265" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A265" t="s">
         <v>291</v>
       </c>
@@ -19792,7 +19792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="307" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A307" t="s">
         <v>593</v>
       </c>
@@ -20842,7 +20842,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="328" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A328" t="s">
         <v>139</v>
       </c>
@@ -22292,7 +22292,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="357" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A357" t="s">
         <v>587</v>
       </c>
@@ -22692,7 +22692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="365" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A365" t="s">
         <v>945</v>
       </c>
@@ -22742,7 +22742,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="366" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A366" t="s">
         <v>949</v>
       </c>
@@ -22842,7 +22842,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="368" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A368" t="s">
         <v>1116</v>
       </c>
@@ -23492,7 +23492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="381" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A381" t="s">
         <v>1123</v>
       </c>
@@ -23542,7 +23542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="382" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="382" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A382" t="s">
         <v>346</v>
       </c>
@@ -24492,7 +24492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="401" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="401" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A401" t="s">
         <v>596</v>
       </c>
@@ -24542,7 +24542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="402" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="402" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A402" t="s">
         <v>866</v>
       </c>
@@ -24942,7 +24942,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="410" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="410" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A410" t="s">
         <v>1104</v>
       </c>
@@ -25142,7 +25142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="414" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="414" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A414" t="s">
         <v>293</v>
       </c>
@@ -26142,7 +26142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="434" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="434" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A434" t="s">
         <v>1142</v>
       </c>
@@ -26192,7 +26192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="435" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="435" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A435" t="s">
         <v>1146</v>
       </c>
@@ -26292,7 +26292,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="437" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="437" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A437" t="s">
         <v>107</v>
       </c>
@@ -26542,7 +26542,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="442" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="442" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A442" t="s">
         <v>113</v>
       </c>
@@ -27142,7 +27142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="454" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="454" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A454" t="s">
         <v>249</v>
       </c>
@@ -27192,7 +27192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="455" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="455" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A455" t="s">
         <v>250</v>
       </c>
@@ -29992,7 +29992,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="511" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="511" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A511" t="s">
         <v>952</v>
       </c>
@@ -30792,7 +30792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="527" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="527" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A527" t="s">
         <v>141</v>
       </c>
@@ -35442,7 +35442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="620" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="620" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A620" t="s">
         <v>1180</v>
       </c>
@@ -35492,7 +35492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="621" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="621" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A621" t="s">
         <v>1180</v>
       </c>
@@ -35546,7 +35546,7 @@
   <autoFilter ref="A1:P621" xr:uid="{6A7ECD2C-6F5B-4E4D-962E-4B55F2FEEDC6}">
     <filterColumn colId="9">
       <filters>
-        <filter val="TYPE_POISON"/>
+        <filter val="TYPE_GHOST"/>
       </filters>
     </filterColumn>
     <filterColumn colId="15">

</xml_diff>

<commit_message>
Update to rival teams through champion fight
</commit_message>
<xml_diff>
--- a/all_generations_pokemon_families.xlsx
+++ b/all_generations_pokemon_families.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3c6863eb3d429a98/Documents/GitHub/pokefirered-expansion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="911" documentId="8_{3DE7B663-32D8-4B09-ACF8-07A7237E0E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C352AAC-F15E-4A9F-A033-83CC755FFAC0}"/>
+  <xr:revisionPtr revIDLastSave="917" documentId="8_{3DE7B663-32D8-4B09-ACF8-07A7237E0E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{63F96B43-E45C-4805-B998-1B4CFBE6DD77}"/>
   <bookViews>
     <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{913F818F-7E2F-42B8-8FB9-B28A63806581}"/>
   </bookViews>
@@ -6042,7 +6042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="32" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>653</v>
       </c>
@@ -7542,7 +7542,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="62" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>122</v>
       </c>
@@ -9142,7 +9142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>942</v>
       </c>
@@ -9192,7 +9192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>946</v>
       </c>
@@ -9942,7 +9942,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="110" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>875</v>
       </c>
@@ -10242,7 +10242,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="116" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>26</v>
       </c>
@@ -10292,7 +10292,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="117" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>502</v>
       </c>
@@ -10342,7 +10342,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="118" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>1027</v>
       </c>
@@ -10492,7 +10492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="121" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>288</v>
       </c>
@@ -10692,7 +10692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="125" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>723</v>
       </c>
@@ -15442,7 +15442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="220" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
         <v>1101</v>
       </c>
@@ -15542,7 +15542,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="222" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
         <v>189</v>
       </c>
@@ -15592,7 +15592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="223" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A223" t="s">
         <v>189</v>
       </c>
@@ -16292,7 +16292,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="237" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A237" t="s">
         <v>410</v>
       </c>
@@ -17192,7 +17192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="255" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A255" t="s">
         <v>656</v>
       </c>
@@ -17392,7 +17392,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="259" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A259" t="s">
         <v>30</v>
       </c>
@@ -17642,7 +17642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="264" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A264" t="s">
         <v>291</v>
       </c>
@@ -17692,7 +17692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="265" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A265" t="s">
         <v>291</v>
       </c>
@@ -17792,7 +17792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="267" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A267" t="s">
         <v>505</v>
       </c>
@@ -17842,7 +17842,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="268" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A268" t="s">
         <v>505</v>
       </c>
@@ -18042,7 +18042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="272" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A272" t="s">
         <v>726</v>
       </c>
@@ -18292,7 +18292,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="277" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
         <v>1030</v>
       </c>
@@ -19792,7 +19792,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="307" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A307" t="s">
         <v>593</v>
       </c>
@@ -22042,7 +22042,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="352" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A352" t="s">
         <v>324</v>
       </c>
@@ -22642,7 +22642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="364" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A364" t="s">
         <v>879</v>
       </c>
@@ -22692,7 +22692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="365" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A365" t="s">
         <v>945</v>
       </c>
@@ -22742,7 +22742,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="366" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A366" t="s">
         <v>949</v>
       </c>
@@ -23342,7 +23342,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="378" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A378" t="s">
         <v>878</v>
       </c>
@@ -23492,7 +23492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="381" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A381" t="s">
         <v>1123</v>
       </c>
@@ -24192,7 +24192,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="395" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="395" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A395" t="s">
         <v>413</v>
       </c>
@@ -24492,7 +24492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="401" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="401" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A401" t="s">
         <v>596</v>
       </c>
@@ -24942,7 +24942,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="410" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="410" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A410" t="s">
         <v>1104</v>
       </c>
@@ -25142,7 +25142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="414" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="414" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A414" t="s">
         <v>293</v>
       </c>
@@ -26592,7 +26592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="443" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="443" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A443" t="s">
         <v>126</v>
       </c>
@@ -29392,7 +29392,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="499" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="499" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A499" t="s">
         <v>449</v>
       </c>
@@ -29992,7 +29992,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="511" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="511" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A511" t="s">
         <v>952</v>
       </c>
@@ -30392,7 +30392,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="519" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="519" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A519" t="s">
         <v>728</v>
       </c>
@@ -30592,7 +30592,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="523" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="523" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A523" t="s">
         <v>32</v>
       </c>
@@ -30642,7 +30642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="524" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="524" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A524" t="s">
         <v>508</v>
       </c>
@@ -30692,7 +30692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="525" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="525" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A525" t="s">
         <v>508</v>
       </c>
@@ -30742,7 +30742,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="526" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="526" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A526" t="s">
         <v>1032</v>
       </c>
@@ -31242,7 +31242,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="536" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="536" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A536" t="s">
         <v>416</v>
       </c>
@@ -31642,7 +31642,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="544" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="544" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A544" t="s">
         <v>193</v>
       </c>
@@ -31692,7 +31692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="545" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="545" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A545" t="s">
         <v>193</v>
       </c>
@@ -32542,7 +32542,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="562" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="562" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A562" t="s">
         <v>483</v>
       </c>
@@ -32692,7 +32692,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="565" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="565" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A565" t="s">
         <v>701</v>
       </c>
@@ -34092,7 +34092,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="593" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="593" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A593" t="s">
         <v>1176</v>
       </c>
@@ -35142,7 +35142,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="614" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="614" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A614" t="s">
         <v>713</v>
       </c>
@@ -35442,7 +35442,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="620" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="620" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A620" t="s">
         <v>1180</v>
       </c>
@@ -35492,7 +35492,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="621" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="621" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A621" t="s">
         <v>1180</v>
       </c>
@@ -35546,7 +35546,7 @@
   <autoFilter ref="A1:P621" xr:uid="{6A7ECD2C-6F5B-4E4D-962E-4B55F2FEEDC6}">
     <filterColumn colId="9">
       <filters>
-        <filter val="TYPE_GHOST"/>
+        <filter val="TYPE_FIRE"/>
       </filters>
     </filterColumn>
     <filterColumn colId="15">

</xml_diff>

<commit_message>
Update to block gyms to enforce game progression order Converting to poryscript throughout
</commit_message>
<xml_diff>
--- a/all_generations_pokemon_families.xlsx
+++ b/all_generations_pokemon_families.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3c6863eb3d429a98/Documents/GitHub/pokefirered-expansion/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Austin\Documents\PokemonDecompBuild\pokefirered-expansion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="917" documentId="8_{3DE7B663-32D8-4B09-ACF8-07A7237E0E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{63F96B43-E45C-4805-B998-1B4CFBE6DD77}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73F2262A-E5B3-4185-A537-AAA20E3A2DD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{913F818F-7E2F-42B8-8FB9-B28A63806581}"/>
   </bookViews>
@@ -4157,10 +4157,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -4992,7 +4988,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="11" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>573</v>
       </c>
@@ -6042,7 +6038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>653</v>
       </c>
@@ -6492,7 +6488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="41" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>1090</v>
       </c>
@@ -6592,7 +6588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="43" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>857</v>
       </c>
@@ -7542,7 +7538,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>122</v>
       </c>
@@ -7692,7 +7688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="65" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>220</v>
       </c>
@@ -8742,7 +8738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="86" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>793</v>
       </c>
@@ -9942,7 +9938,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="110" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>875</v>
       </c>
@@ -10242,7 +10238,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="116" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>26</v>
       </c>
@@ -10292,7 +10288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="117" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>502</v>
       </c>
@@ -10342,7 +10338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="118" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>1027</v>
       </c>
@@ -10642,7 +10638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="124" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>717</v>
       </c>
@@ -10692,7 +10688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="125" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>723</v>
       </c>
@@ -11642,7 +11638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="144" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>15</v>
       </c>
@@ -11692,7 +11688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="145" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>496</v>
       </c>
@@ -11742,7 +11738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="146" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>1021</v>
       </c>
@@ -12242,7 +12238,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="156" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>313</v>
       </c>
@@ -12292,7 +12288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="157" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>313</v>
       </c>
@@ -14192,7 +14188,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="195" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
         <v>1153</v>
       </c>
@@ -14292,7 +14288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="197" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
         <v>893</v>
       </c>
@@ -15542,7 +15538,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="222" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
         <v>189</v>
       </c>
@@ -15592,7 +15588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="223" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A223" t="s">
         <v>189</v>
       </c>
@@ -16292,7 +16288,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="237" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A237" t="s">
         <v>410</v>
       </c>
@@ -16742,7 +16738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="246" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A246" t="s">
         <v>223</v>
       </c>
@@ -17192,7 +17188,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="255" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A255" t="s">
         <v>656</v>
       </c>
@@ -17242,7 +17238,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="256" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A256" t="s">
         <v>860</v>
       </c>
@@ -17342,7 +17338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="258" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A258" t="s">
         <v>22</v>
       </c>
@@ -17392,7 +17388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="259" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A259" t="s">
         <v>30</v>
       </c>
@@ -17742,7 +17738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="266" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A266" t="s">
         <v>499</v>
       </c>
@@ -17792,7 +17788,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="267" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A267" t="s">
         <v>505</v>
       </c>
@@ -17842,7 +17838,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="268" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A268" t="s">
         <v>505</v>
       </c>
@@ -17992,7 +17988,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="271" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A271" t="s">
         <v>720</v>
       </c>
@@ -18042,7 +18038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="272" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A272" t="s">
         <v>726</v>
       </c>
@@ -18242,7 +18238,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="276" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A276" t="s">
         <v>1024</v>
       </c>
@@ -18292,7 +18288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="277" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
         <v>1030</v>
       </c>
@@ -19692,7 +19688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="305" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A305" t="s">
         <v>362</v>
       </c>
@@ -20492,7 +20488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="321" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A321" t="s">
         <v>1093</v>
       </c>
@@ -20792,7 +20788,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="327" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A327" t="s">
         <v>1093</v>
       </c>
@@ -21592,7 +21588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="343" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A343" t="s">
         <v>953</v>
       </c>
@@ -22042,7 +22038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="352" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A352" t="s">
         <v>324</v>
       </c>
@@ -22642,7 +22638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="364" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A364" t="s">
         <v>879</v>
       </c>
@@ -23342,7 +23338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="378" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A378" t="s">
         <v>878</v>
       </c>
@@ -23392,7 +23388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="379" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A379" t="s">
         <v>896</v>
       </c>
@@ -24092,7 +24088,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="393" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="393" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A393" t="s">
         <v>797</v>
       </c>
@@ -24192,7 +24188,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="395" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="395" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A395" t="s">
         <v>413</v>
       </c>
@@ -26242,7 +26238,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="436" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="436" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A436" t="s">
         <v>1156</v>
       </c>
@@ -26592,7 +26588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="443" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="443" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A443" t="s">
         <v>126</v>
       </c>
@@ -26692,7 +26688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="445" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="445" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A445" t="s">
         <v>862</v>
       </c>
@@ -28192,7 +28188,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="475" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="475" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A475" t="s">
         <v>225</v>
       </c>
@@ -28242,7 +28238,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="476" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="476" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A476" t="s">
         <v>317</v>
       </c>
@@ -28292,7 +28288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="477" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="477" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A477" t="s">
         <v>317</v>
       </c>
@@ -28992,7 +28988,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="491" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="491" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A491" t="s">
         <v>24</v>
       </c>
@@ -29392,7 +29388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="499" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="499" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A499" t="s">
         <v>449</v>
       </c>
@@ -29542,7 +29538,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="502" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="502" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A502" t="s">
         <v>452</v>
       </c>
@@ -29642,7 +29638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="504" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="504" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A504" t="s">
         <v>501</v>
       </c>
@@ -30042,7 +30038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="512" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="512" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A512" t="s">
         <v>1026</v>
       </c>
@@ -30342,7 +30338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="518" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="518" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A518" t="s">
         <v>722</v>
       </c>
@@ -30392,7 +30388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="519" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="519" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A519" t="s">
         <v>728</v>
       </c>
@@ -30592,7 +30588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="523" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="523" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A523" t="s">
         <v>32</v>
       </c>
@@ -30642,7 +30638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="524" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="524" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A524" t="s">
         <v>508</v>
       </c>
@@ -30692,7 +30688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="525" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="525" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A525" t="s">
         <v>508</v>
       </c>
@@ -30742,7 +30738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="526" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="526" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A526" t="s">
         <v>1032</v>
       </c>
@@ -30942,7 +30938,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="530" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="530" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A530" t="s">
         <v>366</v>
       </c>
@@ -31242,7 +31238,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="536" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="536" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A536" t="s">
         <v>416</v>
       </c>
@@ -31342,7 +31338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="538" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="538" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A538" t="s">
         <v>576</v>
       </c>
@@ -31642,7 +31638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="544" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="544" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A544" t="s">
         <v>193</v>
       </c>
@@ -31692,7 +31688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="545" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="545" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A545" t="s">
         <v>193</v>
       </c>
@@ -32542,7 +32538,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="562" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="562" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A562" t="s">
         <v>483</v>
       </c>
@@ -32692,7 +32688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="565" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="565" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A565" t="s">
         <v>701</v>
       </c>
@@ -34092,7 +34088,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="593" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="593" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A593" t="s">
         <v>1176</v>
       </c>
@@ -34742,7 +34738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="606" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="606" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A606" t="s">
         <v>1191</v>
       </c>
@@ -34792,7 +34788,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="607" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="607" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A607" t="s">
         <v>1191</v>
       </c>
@@ -35142,7 +35138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="614" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="614" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A614" t="s">
         <v>713</v>
       </c>
@@ -35546,7 +35542,7 @@
   <autoFilter ref="A1:P621" xr:uid="{6A7ECD2C-6F5B-4E4D-962E-4B55F2FEEDC6}">
     <filterColumn colId="9">
       <filters>
-        <filter val="TYPE_FIRE"/>
+        <filter val="TYPE_GRASS"/>
       </filters>
     </filterColumn>
     <filterColumn colId="15">

</xml_diff>

<commit_message>
Updated trainers through rock tunnel
</commit_message>
<xml_diff>
--- a/all_generations_pokemon_families.xlsx
+++ b/all_generations_pokemon_families.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Austin\Documents\PokemonDecompBuild\pokefirered-expansion\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\apetronack\Documents\Projects\pokefirered-expansion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73F2262A-E5B3-4185-A537-AAA20E3A2DD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45660C4E-9CAB-49D2-90D4-FC7E8D0F9FBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{913F818F-7E2F-42B8-8FB9-B28A63806581}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{913F818F-7E2F-42B8-8FB9-B28A63806581}"/>
   </bookViews>
   <sheets>
     <sheet name="all_generations_pokemon_familie" sheetId="1" r:id="rId1"/>
@@ -4988,7 +4988,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>573</v>
       </c>
@@ -6488,7 +6488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>1090</v>
       </c>
@@ -6588,7 +6588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>857</v>
       </c>
@@ -7688,7 +7688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>220</v>
       </c>
@@ -8738,7 +8738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>793</v>
       </c>
@@ -10638,7 +10638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="124" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>717</v>
       </c>
@@ -11638,7 +11638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="144" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>15</v>
       </c>
@@ -11688,7 +11688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="145" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>496</v>
       </c>
@@ -11738,7 +11738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="146" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>1021</v>
       </c>
@@ -12238,7 +12238,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="156" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>313</v>
       </c>
@@ -12288,7 +12288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="157" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>313</v>
       </c>
@@ -14188,7 +14188,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="195" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
         <v>1153</v>
       </c>
@@ -14288,7 +14288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="197" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
         <v>893</v>
       </c>
@@ -16738,7 +16738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="246" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A246" t="s">
         <v>223</v>
       </c>
@@ -17238,7 +17238,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="256" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A256" t="s">
         <v>860</v>
       </c>
@@ -17388,7 +17388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="259" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A259" t="s">
         <v>30</v>
       </c>
@@ -17438,7 +17438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="260" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A260" t="s">
         <v>38</v>
       </c>
@@ -17488,7 +17488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="261" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A261" t="s">
         <v>213</v>
       </c>
@@ -17538,7 +17538,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="262" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A262" t="s">
         <v>217</v>
       </c>
@@ -17588,7 +17588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="263" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A263" t="s">
         <v>217</v>
       </c>
@@ -17638,7 +17638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="264" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A264" t="s">
         <v>291</v>
       </c>
@@ -17688,7 +17688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="265" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A265" t="s">
         <v>291</v>
       </c>
@@ -17788,7 +17788,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="267" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A267" t="s">
         <v>505</v>
       </c>
@@ -17838,7 +17838,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="268" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A268" t="s">
         <v>505</v>
       </c>
@@ -17888,7 +17888,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="269" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A269" t="s">
         <v>512</v>
       </c>
@@ -17938,7 +17938,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="270" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A270" t="s">
         <v>588</v>
       </c>
@@ -18038,7 +18038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="272" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A272" t="s">
         <v>726</v>
       </c>
@@ -18188,7 +18188,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="275" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A275" t="s">
         <v>732</v>
       </c>
@@ -18288,7 +18288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="277" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
         <v>1030</v>
       </c>
@@ -18338,7 +18338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="278" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A278" t="s">
         <v>1036</v>
       </c>
@@ -18388,7 +18388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="279" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A279" t="s">
         <v>708</v>
       </c>
@@ -18438,7 +18438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="280" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A280" t="s">
         <v>971</v>
       </c>
@@ -18488,7 +18488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="281" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A281" t="s">
         <v>1048</v>
       </c>
@@ -18538,7 +18538,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="282" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A282" t="s">
         <v>1128</v>
       </c>
@@ -18588,7 +18588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="283" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A283" t="s">
         <v>679</v>
       </c>
@@ -18638,7 +18638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="284" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A284" t="s">
         <v>489</v>
       </c>
@@ -18688,7 +18688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="285" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A285" t="s">
         <v>995</v>
       </c>
@@ -18738,7 +18738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="286" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A286" t="s">
         <v>518</v>
       </c>
@@ -18788,7 +18788,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="287" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A287" t="s">
         <v>538</v>
       </c>
@@ -18838,7 +18838,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="288" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A288" t="s">
         <v>833</v>
       </c>
@@ -18888,7 +18888,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="289" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A289" t="s">
         <v>618</v>
       </c>
@@ -19288,7 +19288,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="297" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A297" t="s">
         <v>618</v>
       </c>
@@ -19338,7 +19338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="298" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A298" t="s">
         <v>637</v>
       </c>
@@ -19488,7 +19488,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="301" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A301" t="s">
         <v>637</v>
       </c>
@@ -19538,7 +19538,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="302" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A302" t="s">
         <v>637</v>
       </c>
@@ -19588,7 +19588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="303" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A303" t="s">
         <v>637</v>
       </c>
@@ -19638,7 +19638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="304" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A304" t="s">
         <v>838</v>
       </c>
@@ -19738,7 +19738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="306" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A306" t="s">
         <v>432</v>
       </c>
@@ -19788,7 +19788,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="307" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A307" t="s">
         <v>593</v>
       </c>
@@ -19838,7 +19838,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="308" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A308" t="s">
         <v>372</v>
       </c>
@@ -19988,7 +19988,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="311" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A311" t="s">
         <v>801</v>
       </c>
@@ -20038,7 +20038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="312" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A312" t="s">
         <v>95</v>
       </c>
@@ -20088,7 +20088,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="313" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A313" t="s">
         <v>95</v>
       </c>
@@ -20138,7 +20138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="314" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A314" t="s">
         <v>159</v>
       </c>
@@ -20388,7 +20388,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="319" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A319" t="s">
         <v>530</v>
       </c>
@@ -20438,7 +20438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="320" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A320" t="s">
         <v>660</v>
       </c>
@@ -20838,7 +20838,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="328" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A328" t="s">
         <v>139</v>
       </c>
@@ -20888,7 +20888,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="329" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A329" t="s">
         <v>183</v>
       </c>
@@ -20938,7 +20938,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="330" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A330" t="s">
         <v>811</v>
       </c>
@@ -20988,7 +20988,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="331" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A331" t="s">
         <v>389</v>
       </c>
@@ -21038,7 +21038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="332" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A332" t="s">
         <v>389</v>
       </c>
@@ -21088,7 +21088,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="333" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A333" t="s">
         <v>742</v>
       </c>
@@ -21138,7 +21138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="334" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A334" t="s">
         <v>742</v>
       </c>
@@ -21438,7 +21438,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="340" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A340" t="s">
         <v>844</v>
       </c>
@@ -21488,7 +21488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="341" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A341" t="s">
         <v>905</v>
       </c>
@@ -21538,7 +21538,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="342" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A342" t="s">
         <v>907</v>
       </c>
@@ -21638,7 +21638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="344" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A344" t="s">
         <v>155</v>
       </c>
@@ -21988,7 +21988,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="351" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A351" t="s">
         <v>324</v>
       </c>
@@ -22038,7 +22038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="352" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A352" t="s">
         <v>324</v>
       </c>
@@ -22088,7 +22088,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="353" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A353" t="s">
         <v>273</v>
       </c>
@@ -22138,7 +22138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="354" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A354" t="s">
         <v>738</v>
       </c>
@@ -22188,7 +22188,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="355" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A355" t="s">
         <v>884</v>
       </c>
@@ -22238,7 +22238,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="356" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A356" t="s">
         <v>584</v>
       </c>
@@ -22288,7 +22288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="357" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A357" t="s">
         <v>587</v>
       </c>
@@ -22488,7 +22488,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="361" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A361" t="s">
         <v>601</v>
       </c>
@@ -22538,7 +22538,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="362" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A362" t="s">
         <v>774</v>
       </c>
@@ -22588,7 +22588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="363" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A363" t="s">
         <v>848</v>
       </c>
@@ -22638,7 +22638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="364" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A364" t="s">
         <v>879</v>
       </c>
@@ -22688,7 +22688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="365" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A365" t="s">
         <v>945</v>
       </c>
@@ -22738,7 +22738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="366" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A366" t="s">
         <v>949</v>
       </c>
@@ -22788,7 +22788,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="367" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A367" t="s">
         <v>61</v>
       </c>
@@ -22838,7 +22838,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="368" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A368" t="s">
         <v>1116</v>
       </c>
@@ -22888,7 +22888,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="369" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A369" t="s">
         <v>259</v>
       </c>
@@ -22938,7 +22938,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="370" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A370" t="s">
         <v>259</v>
       </c>
@@ -22988,7 +22988,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="371" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="371" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A371" t="s">
         <v>534</v>
       </c>
@@ -23038,7 +23038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="372" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A372" t="s">
         <v>680</v>
       </c>
@@ -23088,7 +23088,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="373" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A373" t="s">
         <v>916</v>
       </c>
@@ -23138,7 +23138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="374" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A374" t="s">
         <v>1108</v>
       </c>
@@ -23188,7 +23188,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="375" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A375" t="s">
         <v>1185</v>
       </c>
@@ -23238,7 +23238,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="376" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A376" t="s">
         <v>822</v>
       </c>
@@ -23288,7 +23288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="377" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A377" t="s">
         <v>350</v>
       </c>
@@ -23338,7 +23338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="378" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A378" t="s">
         <v>878</v>
       </c>
@@ -23438,7 +23438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="380" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A380" t="s">
         <v>1044</v>
       </c>
@@ -23488,7 +23488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="381" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A381" t="s">
         <v>1123</v>
       </c>
@@ -23538,7 +23538,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="382" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="382" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A382" t="s">
         <v>346</v>
       </c>
@@ -23588,7 +23588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="383" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="383" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A383" t="s">
         <v>367</v>
       </c>
@@ -23638,7 +23638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="384" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="384" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A384" t="s">
         <v>406</v>
       </c>
@@ -23688,7 +23688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="385" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="385" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A385" t="s">
         <v>557</v>
       </c>
@@ -23738,7 +23738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="386" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="386" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A386" t="s">
         <v>697</v>
       </c>
@@ -24138,7 +24138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="394" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="394" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A394" t="s">
         <v>302</v>
       </c>
@@ -24188,7 +24188,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="395" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="395" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A395" t="s">
         <v>413</v>
       </c>
@@ -24388,7 +24388,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="399" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="399" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A399" t="s">
         <v>466</v>
       </c>
@@ -24438,7 +24438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="400" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="400" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A400" t="s">
         <v>470</v>
       </c>
@@ -24488,7 +24488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="401" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="401" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A401" t="s">
         <v>596</v>
       </c>
@@ -24538,7 +24538,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="402" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="402" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A402" t="s">
         <v>866</v>
       </c>
@@ -24588,7 +24588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="403" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="403" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A403" t="s">
         <v>924</v>
       </c>
@@ -24638,7 +24638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="404" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="404" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A404" t="s">
         <v>928</v>
       </c>
@@ -24688,7 +24688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="405" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="405" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A405" t="s">
         <v>1062</v>
       </c>
@@ -24738,7 +24738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="406" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="406" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A406" t="s">
         <v>1066</v>
       </c>
@@ -24788,7 +24788,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="407" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="407" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A407" t="s">
         <v>1089</v>
       </c>
@@ -24938,7 +24938,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="410" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="410" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A410" t="s">
         <v>1104</v>
       </c>
@@ -24988,7 +24988,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="411" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="411" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A411" t="s">
         <v>89</v>
       </c>
@@ -25038,7 +25038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="412" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="412" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A412" t="s">
         <v>89</v>
       </c>
@@ -25088,7 +25088,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="413" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="413" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A413" t="s">
         <v>178</v>
       </c>
@@ -25138,7 +25138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="414" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="414" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A414" t="s">
         <v>293</v>
       </c>
@@ -25188,7 +25188,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="415" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="415" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A415" t="s">
         <v>392</v>
       </c>
@@ -25238,7 +25238,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="416" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="416" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A416" t="s">
         <v>392</v>
       </c>
@@ -25288,7 +25288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="417" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="417" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A417" t="s">
         <v>397</v>
       </c>
@@ -25338,7 +25338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="418" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="418" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A418" t="s">
         <v>398</v>
       </c>
@@ -25388,7 +25388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="419" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="419" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A419" t="s">
         <v>545</v>
       </c>
@@ -25438,7 +25438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="420" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="420" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A420" t="s">
         <v>609</v>
       </c>
@@ -25488,7 +25488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="421" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="421" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A421" t="s">
         <v>635</v>
       </c>
@@ -25538,7 +25538,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="422" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="422" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A422" t="s">
         <v>685</v>
       </c>
@@ -25588,7 +25588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="423" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="423" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A423" t="s">
         <v>689</v>
       </c>
@@ -25938,7 +25938,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="430" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="430" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A430" t="s">
         <v>764</v>
       </c>
@@ -25988,7 +25988,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="431" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="431" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A431" t="s">
         <v>874</v>
       </c>
@@ -26038,7 +26038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="432" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="432" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A432" t="s">
         <v>920</v>
       </c>
@@ -26088,7 +26088,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="433" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="433" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A433" t="s">
         <v>1120</v>
       </c>
@@ -26138,7 +26138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="434" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="434" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A434" t="s">
         <v>1142</v>
       </c>
@@ -26188,7 +26188,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="435" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="435" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A435" t="s">
         <v>1146</v>
       </c>
@@ -26288,7 +26288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="437" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="437" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A437" t="s">
         <v>107</v>
       </c>
@@ -26538,7 +26538,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="442" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="442" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A442" t="s">
         <v>113</v>
       </c>
@@ -26588,7 +26588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="443" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="443" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A443" t="s">
         <v>126</v>
       </c>
@@ -26638,7 +26638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="444" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="444" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A444" t="s">
         <v>633</v>
       </c>
@@ -26738,7 +26738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="446" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="446" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A446" t="s">
         <v>205</v>
       </c>
@@ -26888,7 +26888,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="449" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="449" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A449" t="s">
         <v>206</v>
       </c>
@@ -26938,7 +26938,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="450" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="450" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A450" t="s">
         <v>235</v>
       </c>
@@ -26988,7 +26988,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="451" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="451" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A451" t="s">
         <v>235</v>
       </c>
@@ -27038,7 +27038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="452" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="452" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A452" t="s">
         <v>249</v>
       </c>
@@ -27088,7 +27088,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="453" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="453" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A453" t="s">
         <v>250</v>
       </c>
@@ -27138,7 +27138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="454" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="454" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A454" t="s">
         <v>249</v>
       </c>
@@ -27188,7 +27188,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="455" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="455" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A455" t="s">
         <v>250</v>
       </c>
@@ -27288,7 +27288,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="457" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="457" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A457" t="s">
         <v>298</v>
       </c>
@@ -27338,7 +27338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="458" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="458" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A458" t="s">
         <v>641</v>
       </c>
@@ -27388,7 +27388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="459" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="459" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A459" t="s">
         <v>644</v>
       </c>
@@ -27438,7 +27438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="460" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="460" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A460" t="s">
         <v>900</v>
       </c>
@@ -27488,7 +27488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="461" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="461" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A461" t="s">
         <v>966</v>
       </c>
@@ -27538,7 +27538,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="462" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="462" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A462" t="s">
         <v>967</v>
       </c>
@@ -27588,7 +27588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="463" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="463" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A463" t="s">
         <v>980</v>
       </c>
@@ -27738,7 +27738,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="466" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="466" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A466" t="s">
         <v>981</v>
       </c>
@@ -27788,7 +27788,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="467" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="467" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A467" t="s">
         <v>229</v>
       </c>
@@ -27938,7 +27938,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="470" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="470" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A470" t="s">
         <v>459</v>
       </c>
@@ -27988,7 +27988,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="471" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="471" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A471" t="s">
         <v>471</v>
       </c>
@@ -28038,7 +28038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="472" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="472" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A472" t="s">
         <v>592</v>
       </c>
@@ -28088,7 +28088,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="473" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="473" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A473" t="s">
         <v>787</v>
       </c>
@@ -28138,7 +28138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="474" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="474" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A474" t="s">
         <v>788</v>
       </c>
@@ -28338,7 +28338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="478" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="478" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A478" t="s">
         <v>383</v>
       </c>
@@ -28388,7 +28388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="479" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="479" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A479" t="s">
         <v>391</v>
       </c>
@@ -28438,7 +28438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="480" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="480" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A480" t="s">
         <v>551</v>
       </c>
@@ -28738,7 +28738,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="486" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="486" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A486" t="s">
         <v>605</v>
       </c>
@@ -28788,7 +28788,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="487" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="487" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A487" t="s">
         <v>746</v>
       </c>
@@ -28838,7 +28838,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="488" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="488" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A488" t="s">
         <v>818</v>
       </c>
@@ -28888,7 +28888,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="489" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="489" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A489" t="s">
         <v>892</v>
       </c>
@@ -28938,7 +28938,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="490" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="490" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A490" t="s">
         <v>1058</v>
       </c>
@@ -29188,7 +29188,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="495" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="495" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A495" t="s">
         <v>219</v>
       </c>
@@ -29238,7 +29238,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="496" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="496" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A496" t="s">
         <v>287</v>
       </c>
@@ -29288,7 +29288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="497" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="497" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A497" t="s">
         <v>447</v>
       </c>
@@ -29338,7 +29338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="498" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="498" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A498" t="s">
         <v>448</v>
       </c>
@@ -29388,7 +29388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="499" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="499" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A499" t="s">
         <v>449</v>
       </c>
@@ -29438,7 +29438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="500" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="500" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A500" t="s">
         <v>450</v>
       </c>
@@ -29488,7 +29488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="501" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="501" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A501" t="s">
         <v>451</v>
       </c>
@@ -29588,7 +29588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="503" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="503" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A503" t="s">
         <v>453</v>
       </c>
@@ -29688,7 +29688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="505" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="505" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A505" t="s">
         <v>622</v>
       </c>
@@ -29988,7 +29988,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="511" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="511" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A511" t="s">
         <v>952</v>
       </c>
@@ -30088,7 +30088,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="513" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="513" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A513" t="s">
         <v>1134</v>
       </c>
@@ -30138,7 +30138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="514" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="514" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A514" t="s">
         <v>1138</v>
       </c>
@@ -30188,7 +30188,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="515" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="515" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A515" t="s">
         <v>40</v>
       </c>
@@ -30238,7 +30238,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="516" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="516" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A516" t="s">
         <v>514</v>
       </c>
@@ -30288,7 +30288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="517" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="517" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A517" t="s">
         <v>662</v>
       </c>
@@ -30388,7 +30388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="519" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="519" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A519" t="s">
         <v>728</v>
       </c>
@@ -30438,7 +30438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="520" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="520" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A520" t="s">
         <v>840</v>
       </c>
@@ -30488,7 +30488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="521" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="521" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A521" t="s">
         <v>973</v>
       </c>
@@ -30538,7 +30538,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="522" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="522" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A522" t="s">
         <v>1038</v>
       </c>
@@ -30588,7 +30588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="523" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="523" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A523" t="s">
         <v>32</v>
       </c>
@@ -30638,7 +30638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="524" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="524" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A524" t="s">
         <v>508</v>
       </c>
@@ -30688,7 +30688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="525" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="525" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A525" t="s">
         <v>508</v>
       </c>
@@ -30738,7 +30738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="526" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="526" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A526" t="s">
         <v>1032</v>
       </c>
@@ -30788,7 +30788,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="527" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="527" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A527" t="s">
         <v>141</v>
       </c>
@@ -30838,7 +30838,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="528" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="528" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A528" t="s">
         <v>187</v>
       </c>
@@ -30888,7 +30888,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="529" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="529" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A529" t="s">
         <v>353</v>
       </c>
@@ -30988,7 +30988,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="531" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="531" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A531" t="s">
         <v>428</v>
       </c>
@@ -31038,7 +31038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="532" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="532" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A532" t="s">
         <v>462</v>
       </c>
@@ -31088,7 +31088,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="533" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="533" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A533" t="s">
         <v>734</v>
       </c>
@@ -31138,7 +31138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="534" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="534" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A534" t="s">
         <v>375</v>
       </c>
@@ -31188,7 +31188,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="535" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="535" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A535" t="s">
         <v>409</v>
       </c>
@@ -31238,7 +31238,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="536" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="536" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A536" t="s">
         <v>416</v>
       </c>
@@ -31288,7 +31288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="537" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="537" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A537" t="s">
         <v>476</v>
       </c>
@@ -31388,7 +31388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="539" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="539" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A539" t="s">
         <v>934</v>
       </c>
@@ -31438,7 +31438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="540" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="540" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A540" t="s">
         <v>263</v>
       </c>
@@ -31588,7 +31588,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="543" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="543" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A543" t="s">
         <v>541</v>
       </c>
@@ -31638,7 +31638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="544" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="544" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A544" t="s">
         <v>193</v>
       </c>
@@ -31688,7 +31688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="545" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="545" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A545" t="s">
         <v>193</v>
       </c>
@@ -31738,7 +31738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="546" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="546" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A546" t="s">
         <v>477</v>
       </c>
@@ -31788,7 +31788,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="547" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="547" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A547" t="s">
         <v>477</v>
       </c>
@@ -31838,7 +31838,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="548" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="548" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A548" t="s">
         <v>480</v>
       </c>
@@ -31888,7 +31888,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="549" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="549" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A549" t="s">
         <v>480</v>
       </c>
@@ -32538,7 +32538,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="562" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="562" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A562" t="s">
         <v>483</v>
       </c>
@@ -32588,7 +32588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="563" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="563" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A563" t="s">
         <v>483</v>
       </c>
@@ -32638,7 +32638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="564" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="564" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A564" t="s">
         <v>699</v>
       </c>
@@ -32688,7 +32688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="565" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="565" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A565" t="s">
         <v>701</v>
       </c>
@@ -32738,7 +32738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="566" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="566" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A566" t="s">
         <v>703</v>
       </c>
@@ -32988,7 +32988,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="571" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="571" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A571" t="s">
         <v>998</v>
       </c>
@@ -33038,7 +33038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="572" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="572" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A572" t="s">
         <v>1000</v>
       </c>
@@ -33088,7 +33088,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="573" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="573" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A573" t="s">
         <v>1002</v>
       </c>
@@ -33138,7 +33138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="574" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="574" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A574" t="s">
         <v>1164</v>
       </c>
@@ -33288,7 +33288,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="577" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="577" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A577" t="s">
         <v>1166</v>
       </c>
@@ -33338,7 +33338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="578" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="578" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A578" t="s">
         <v>1168</v>
       </c>
@@ -33388,7 +33388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="579" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="579" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A579" t="s">
         <v>491</v>
       </c>
@@ -33438,7 +33438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="580" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="580" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A580" t="s">
         <v>494</v>
       </c>
@@ -33538,7 +33538,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="582" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="582" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A582" t="s">
         <v>710</v>
       </c>
@@ -33588,7 +33588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="583" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="583" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A583" t="s">
         <v>715</v>
       </c>
@@ -33638,7 +33638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="584" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="584" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A584" t="s">
         <v>997</v>
       </c>
@@ -33688,7 +33688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="585" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="585" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A585" t="s">
         <v>1004</v>
       </c>
@@ -33738,7 +33738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="586" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="586" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A586" t="s">
         <v>1006</v>
       </c>
@@ -33788,7 +33788,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="587" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="587" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A587" t="s">
         <v>1014</v>
       </c>
@@ -33838,7 +33838,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="588" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="588" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A588" t="s">
         <v>1016</v>
       </c>
@@ -33888,7 +33888,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="589" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="589" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A589" t="s">
         <v>1016</v>
       </c>
@@ -33938,7 +33938,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="590" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="590" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A590" t="s">
         <v>1016</v>
       </c>
@@ -33988,7 +33988,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="591" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="591" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A591" t="s">
         <v>1016</v>
       </c>
@@ -34038,7 +34038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="592" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="592" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A592" t="s">
         <v>1130</v>
       </c>
@@ -34088,7 +34088,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="593" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="593" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A593" t="s">
         <v>1176</v>
       </c>
@@ -34288,7 +34288,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="597" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="597" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A597" t="s">
         <v>1183</v>
       </c>
@@ -34338,7 +34338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="598" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="598" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A598" t="s">
         <v>1187</v>
       </c>
@@ -34688,7 +34688,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="605" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="605" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A605" t="s">
         <v>1189</v>
       </c>
@@ -34838,7 +34838,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="608" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="608" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A608" t="s">
         <v>803</v>
       </c>
@@ -34888,7 +34888,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="609" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="609" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A609" t="s">
         <v>1008</v>
       </c>
@@ -34938,7 +34938,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="610" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="610" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A610" t="s">
         <v>1010</v>
       </c>
@@ -34988,7 +34988,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="611" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="611" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A611" t="s">
         <v>1178</v>
       </c>
@@ -35038,7 +35038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="612" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="612" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A612" t="s">
         <v>492</v>
       </c>
@@ -35088,7 +35088,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="613" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="613" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A613" t="s">
         <v>711</v>
       </c>
@@ -35138,7 +35138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="614" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="614" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A614" t="s">
         <v>713</v>
       </c>
@@ -35188,7 +35188,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="615" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="615" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A615" t="s">
         <v>1012</v>
       </c>
@@ -35238,7 +35238,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="616" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="616" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A616" t="s">
         <v>1170</v>
       </c>
@@ -35288,7 +35288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="617" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="617" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A617" t="s">
         <v>1170</v>
       </c>
@@ -35338,7 +35338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="618" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="618" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A618" t="s">
         <v>1173</v>
       </c>
@@ -35388,7 +35388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="619" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="619" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A619" t="s">
         <v>1173</v>
       </c>
@@ -35438,7 +35438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="620" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="620" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A620" t="s">
         <v>1180</v>
       </c>
@@ -35488,7 +35488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="621" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="621" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A621" t="s">
         <v>1180</v>
       </c>
@@ -35540,10 +35540,10 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:P621" xr:uid="{6A7ECD2C-6F5B-4E4D-962E-4B55F2FEEDC6}">
-    <filterColumn colId="9">
-      <filters>
-        <filter val="TYPE_GRASS"/>
-      </filters>
+    <filterColumn colId="8">
+      <customFilters>
+        <customFilter operator="greaterThan" val="400"/>
+      </customFilters>
     </filterColumn>
     <filterColumn colId="15">
       <filters>

</xml_diff>

<commit_message>
Initial route 12 trainer updates
</commit_message>
<xml_diff>
--- a/all_generations_pokemon_families.xlsx
+++ b/all_generations_pokemon_families.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\apetronack\Documents\Projects\pokefirered-expansion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EBE7E01-8550-484B-BFAD-D853392BDD24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{640D09F9-2BEB-4A1E-ABBB-ACCC28723074}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{913F818F-7E2F-42B8-8FB9-B28A63806581}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{913F818F-7E2F-42B8-8FB9-B28A63806581}"/>
   </bookViews>
   <sheets>
     <sheet name="all_generations_pokemon_familie" sheetId="1" r:id="rId1"/>
@@ -17338,7 +17338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="258" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A258" t="s">
         <v>22</v>
       </c>
@@ -17388,7 +17388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="259" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A259" t="s">
         <v>30</v>
       </c>
@@ -17488,7 +17488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="261" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A261" t="s">
         <v>213</v>
       </c>
@@ -17538,7 +17538,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="262" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A262" t="s">
         <v>217</v>
       </c>
@@ -17588,7 +17588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="263" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A263" t="s">
         <v>217</v>
       </c>
@@ -17638,7 +17638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="264" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A264" t="s">
         <v>291</v>
       </c>
@@ -17688,7 +17688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="265" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A265" t="s">
         <v>291</v>
       </c>
@@ -17738,7 +17738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="266" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A266" t="s">
         <v>499</v>
       </c>
@@ -17788,7 +17788,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="267" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A267" t="s">
         <v>505</v>
       </c>
@@ -17838,7 +17838,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="268" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A268" t="s">
         <v>505</v>
       </c>
@@ -17938,7 +17938,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="270" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A270" t="s">
         <v>588</v>
       </c>
@@ -17988,7 +17988,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="271" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A271" t="s">
         <v>720</v>
       </c>
@@ -18038,7 +18038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="272" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A272" t="s">
         <v>726</v>
       </c>
@@ -18238,7 +18238,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="276" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A276" t="s">
         <v>1024</v>
       </c>
@@ -18288,7 +18288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="277" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
         <v>1030</v>
       </c>
@@ -18388,7 +18388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="279" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A279" t="s">
         <v>708</v>
       </c>
@@ -18438,7 +18438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="280" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A280" t="s">
         <v>971</v>
       </c>
@@ -18488,7 +18488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="281" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A281" t="s">
         <v>1048</v>
       </c>
@@ -18538,7 +18538,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="282" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A282" t="s">
         <v>1128</v>
       </c>
@@ -18638,7 +18638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="284" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A284" t="s">
         <v>489</v>
       </c>
@@ -18688,7 +18688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="285" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A285" t="s">
         <v>995</v>
       </c>
@@ -18738,7 +18738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="286" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A286" t="s">
         <v>518</v>
       </c>
@@ -18788,7 +18788,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="287" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A287" t="s">
         <v>538</v>
       </c>
@@ -18838,7 +18838,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="288" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A288" t="s">
         <v>833</v>
       </c>
@@ -18888,7 +18888,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="289" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A289" t="s">
         <v>618</v>
       </c>
@@ -19288,7 +19288,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="297" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A297" t="s">
         <v>618</v>
       </c>
@@ -19338,7 +19338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="298" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A298" t="s">
         <v>637</v>
       </c>
@@ -19488,7 +19488,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="301" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A301" t="s">
         <v>637</v>
       </c>
@@ -19538,7 +19538,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="302" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A302" t="s">
         <v>637</v>
       </c>
@@ -19588,7 +19588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="303" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A303" t="s">
         <v>637</v>
       </c>
@@ -19638,7 +19638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="304" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A304" t="s">
         <v>838</v>
       </c>
@@ -19688,7 +19688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="305" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A305" t="s">
         <v>362</v>
       </c>
@@ -19738,7 +19738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="306" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A306" t="s">
         <v>432</v>
       </c>
@@ -19788,7 +19788,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="307" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A307" t="s">
         <v>593</v>
       </c>
@@ -19988,7 +19988,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="311" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A311" t="s">
         <v>801</v>
       </c>
@@ -20038,7 +20038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="312" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A312" t="s">
         <v>95</v>
       </c>
@@ -20088,7 +20088,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="313" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A313" t="s">
         <v>95</v>
       </c>
@@ -20138,7 +20138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="314" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A314" t="s">
         <v>159</v>
       </c>
@@ -20388,7 +20388,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="319" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A319" t="s">
         <v>530</v>
       </c>
@@ -20438,7 +20438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="320" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A320" t="s">
         <v>660</v>
       </c>
@@ -20488,7 +20488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="321" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A321" t="s">
         <v>1093</v>
       </c>
@@ -20788,7 +20788,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="327" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A327" t="s">
         <v>1093</v>
       </c>
@@ -20838,7 +20838,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="328" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A328" t="s">
         <v>139</v>
       </c>
@@ -20888,7 +20888,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="329" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A329" t="s">
         <v>183</v>
       </c>
@@ -20938,7 +20938,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="330" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A330" t="s">
         <v>811</v>
       </c>
@@ -20988,7 +20988,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="331" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A331" t="s">
         <v>389</v>
       </c>
@@ -21038,7 +21038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="332" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A332" t="s">
         <v>389</v>
       </c>
@@ -21088,7 +21088,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="333" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A333" t="s">
         <v>742</v>
       </c>
@@ -21138,7 +21138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="334" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A334" t="s">
         <v>742</v>
       </c>
@@ -21438,7 +21438,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="340" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A340" t="s">
         <v>844</v>
       </c>
@@ -21488,7 +21488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="341" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A341" t="s">
         <v>905</v>
       </c>
@@ -21538,7 +21538,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="342" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A342" t="s">
         <v>907</v>
       </c>
@@ -21588,7 +21588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="343" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A343" t="s">
         <v>953</v>
       </c>
@@ -21638,7 +21638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="344" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A344" t="s">
         <v>155</v>
       </c>
@@ -21988,7 +21988,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="351" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A351" t="s">
         <v>324</v>
       </c>
@@ -22038,7 +22038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="352" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A352" t="s">
         <v>324</v>
       </c>
@@ -22088,7 +22088,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="353" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A353" t="s">
         <v>273</v>
       </c>
@@ -22138,7 +22138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="354" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A354" t="s">
         <v>738</v>
       </c>
@@ -22188,7 +22188,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="355" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A355" t="s">
         <v>884</v>
       </c>
@@ -22288,7 +22288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="357" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A357" t="s">
         <v>587</v>
       </c>
@@ -22488,7 +22488,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="361" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A361" t="s">
         <v>601</v>
       </c>
@@ -22538,7 +22538,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="362" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A362" t="s">
         <v>774</v>
       </c>
@@ -22588,7 +22588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="363" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A363" t="s">
         <v>848</v>
       </c>
@@ -22638,7 +22638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="364" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A364" t="s">
         <v>879</v>
       </c>
@@ -22688,7 +22688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="365" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A365" t="s">
         <v>945</v>
       </c>
@@ -22738,7 +22738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="366" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A366" t="s">
         <v>949</v>
       </c>
@@ -22788,7 +22788,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="367" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A367" t="s">
         <v>61</v>
       </c>
@@ -22838,7 +22838,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="368" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A368" t="s">
         <v>1116</v>
       </c>
@@ -22888,7 +22888,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="369" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A369" t="s">
         <v>259</v>
       </c>
@@ -22938,7 +22938,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="370" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A370" t="s">
         <v>259</v>
       </c>
@@ -23038,7 +23038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="372" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A372" t="s">
         <v>680</v>
       </c>
@@ -23138,7 +23138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="374" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A374" t="s">
         <v>1108</v>
       </c>
@@ -23238,7 +23238,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="376" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A376" t="s">
         <v>822</v>
       </c>
@@ -23288,7 +23288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="377" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A377" t="s">
         <v>350</v>
       </c>
@@ -23338,7 +23338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="378" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A378" t="s">
         <v>878</v>
       </c>
@@ -23388,7 +23388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="379" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A379" t="s">
         <v>896</v>
       </c>
@@ -23438,7 +23438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="380" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A380" t="s">
         <v>1044</v>
       </c>
@@ -23488,7 +23488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="381" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A381" t="s">
         <v>1123</v>
       </c>
@@ -23538,7 +23538,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="382" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="382" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A382" t="s">
         <v>346</v>
       </c>
@@ -23588,7 +23588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="383" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="383" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A383" t="s">
         <v>367</v>
       </c>
@@ -23638,7 +23638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="384" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="384" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A384" t="s">
         <v>406</v>
       </c>
@@ -23738,7 +23738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="386" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="386" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A386" t="s">
         <v>697</v>
       </c>
@@ -24088,7 +24088,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="393" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="393" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A393" t="s">
         <v>797</v>
       </c>
@@ -24138,7 +24138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="394" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="394" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A394" t="s">
         <v>302</v>
       </c>
@@ -24188,7 +24188,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="395" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="395" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A395" t="s">
         <v>413</v>
       </c>
@@ -24388,7 +24388,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="399" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="399" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A399" t="s">
         <v>466</v>
       </c>
@@ -24438,7 +24438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="400" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="400" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A400" t="s">
         <v>470</v>
       </c>
@@ -24488,7 +24488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="401" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="401" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A401" t="s">
         <v>596</v>
       </c>
@@ -24538,7 +24538,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="402" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="402" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A402" t="s">
         <v>866</v>
       </c>
@@ -24588,7 +24588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="403" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="403" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A403" t="s">
         <v>924</v>
       </c>
@@ -24638,7 +24638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="404" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="404" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A404" t="s">
         <v>928</v>
       </c>
@@ -24688,7 +24688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="405" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="405" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A405" t="s">
         <v>1062</v>
       </c>
@@ -24738,7 +24738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="406" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="406" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A406" t="s">
         <v>1066</v>
       </c>
@@ -24938,7 +24938,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="410" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="410" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A410" t="s">
         <v>1104</v>
       </c>
@@ -24988,7 +24988,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="411" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="411" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A411" t="s">
         <v>89</v>
       </c>
@@ -25038,7 +25038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="412" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="412" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A412" t="s">
         <v>89</v>
       </c>
@@ -25138,7 +25138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="414" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="414" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A414" t="s">
         <v>293</v>
       </c>
@@ -25188,7 +25188,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="415" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="415" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A415" t="s">
         <v>392</v>
       </c>
@@ -25238,7 +25238,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="416" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="416" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A416" t="s">
         <v>392</v>
       </c>
@@ -25288,7 +25288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="417" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="417" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A417" t="s">
         <v>397</v>
       </c>
@@ -25338,7 +25338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="418" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="418" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A418" t="s">
         <v>398</v>
       </c>
@@ -25388,7 +25388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="419" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="419" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A419" t="s">
         <v>545</v>
       </c>
@@ -25438,7 +25438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="420" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="420" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A420" t="s">
         <v>609</v>
       </c>
@@ -25488,7 +25488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="421" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="421" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A421" t="s">
         <v>635</v>
       </c>
@@ -25538,7 +25538,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="422" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="422" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A422" t="s">
         <v>685</v>
       </c>
@@ -25588,7 +25588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="423" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="423" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A423" t="s">
         <v>689</v>
       </c>
@@ -26038,7 +26038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="432" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="432" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A432" t="s">
         <v>920</v>
       </c>
@@ -26088,7 +26088,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="433" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="433" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A433" t="s">
         <v>1120</v>
       </c>
@@ -26138,7 +26138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="434" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="434" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A434" t="s">
         <v>1142</v>
       </c>
@@ -26188,7 +26188,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="435" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="435" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A435" t="s">
         <v>1146</v>
       </c>
@@ -26238,7 +26238,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="436" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="436" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A436" t="s">
         <v>1156</v>
       </c>
@@ -26288,7 +26288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="437" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="437" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A437" t="s">
         <v>107</v>
       </c>
@@ -26538,7 +26538,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="442" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="442" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A442" t="s">
         <v>113</v>
       </c>
@@ -26588,7 +26588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="443" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="443" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A443" t="s">
         <v>126</v>
       </c>
@@ -26638,7 +26638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="444" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="444" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A444" t="s">
         <v>633</v>
       </c>
@@ -26688,7 +26688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="445" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="445" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A445" t="s">
         <v>862</v>
       </c>
@@ -26938,7 +26938,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="450" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="450" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A450" t="s">
         <v>235</v>
       </c>
@@ -26988,7 +26988,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="451" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="451" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A451" t="s">
         <v>235</v>
       </c>
@@ -27138,7 +27138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="454" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="454" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A454" t="s">
         <v>249</v>
       </c>
@@ -27188,7 +27188,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="455" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="455" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A455" t="s">
         <v>250</v>
       </c>
@@ -27288,7 +27288,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="457" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="457" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A457" t="s">
         <v>298</v>
       </c>
@@ -27338,7 +27338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="458" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="458" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A458" t="s">
         <v>641</v>
       </c>
@@ -27388,7 +27388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="459" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="459" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A459" t="s">
         <v>644</v>
       </c>
@@ -27438,7 +27438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="460" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="460" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A460" t="s">
         <v>900</v>
       </c>
@@ -27488,7 +27488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="461" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="461" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A461" t="s">
         <v>966</v>
       </c>
@@ -27538,7 +27538,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="462" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="462" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A462" t="s">
         <v>967</v>
       </c>
@@ -27938,7 +27938,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="470" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="470" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A470" t="s">
         <v>459</v>
       </c>
@@ -27988,7 +27988,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="471" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="471" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A471" t="s">
         <v>471</v>
       </c>
@@ -28038,7 +28038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="472" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="472" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A472" t="s">
         <v>592</v>
       </c>
@@ -28088,7 +28088,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="473" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="473" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A473" t="s">
         <v>787</v>
       </c>
@@ -28138,7 +28138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="474" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="474" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A474" t="s">
         <v>788</v>
       </c>
@@ -28188,7 +28188,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="475" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="475" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A475" t="s">
         <v>225</v>
       </c>
@@ -28238,7 +28238,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="476" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="476" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A476" t="s">
         <v>317</v>
       </c>
@@ -28288,7 +28288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="477" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="477" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A477" t="s">
         <v>317</v>
       </c>
@@ -28388,7 +28388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="479" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="479" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A479" t="s">
         <v>391</v>
       </c>
@@ -28438,7 +28438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="480" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="480" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A480" t="s">
         <v>551</v>
       </c>
@@ -28738,7 +28738,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="486" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="486" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A486" t="s">
         <v>605</v>
       </c>
@@ -28788,7 +28788,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="487" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="487" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A487" t="s">
         <v>746</v>
       </c>
@@ -28838,7 +28838,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="488" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="488" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A488" t="s">
         <v>818</v>
       </c>
@@ -28888,7 +28888,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="489" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="489" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A489" t="s">
         <v>892</v>
       </c>
@@ -28938,7 +28938,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="490" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="490" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A490" t="s">
         <v>1058</v>
       </c>
@@ -28988,7 +28988,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="491" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="491" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A491" t="s">
         <v>24</v>
       </c>
@@ -29188,7 +29188,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="495" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="495" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A495" t="s">
         <v>219</v>
       </c>
@@ -29338,7 +29338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="498" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="498" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A498" t="s">
         <v>448</v>
       </c>
@@ -29388,7 +29388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="499" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="499" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A499" t="s">
         <v>449</v>
       </c>
@@ -29438,7 +29438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="500" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="500" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A500" t="s">
         <v>450</v>
       </c>
@@ -29488,7 +29488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="501" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="501" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A501" t="s">
         <v>451</v>
       </c>
@@ -29538,7 +29538,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="502" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="502" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A502" t="s">
         <v>452</v>
       </c>
@@ -29588,7 +29588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="503" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="503" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A503" t="s">
         <v>453</v>
       </c>
@@ -29638,7 +29638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="504" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="504" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A504" t="s">
         <v>501</v>
       </c>
@@ -29688,7 +29688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="505" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="505" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A505" t="s">
         <v>622</v>
       </c>
@@ -29988,7 +29988,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="511" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="511" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A511" t="s">
         <v>952</v>
       </c>
@@ -30038,7 +30038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="512" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="512" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A512" t="s">
         <v>1026</v>
       </c>
@@ -30088,7 +30088,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="513" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="513" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A513" t="s">
         <v>1134</v>
       </c>
@@ -30138,7 +30138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="514" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="514" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A514" t="s">
         <v>1138</v>
       </c>
@@ -30288,7 +30288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="517" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="517" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A517" t="s">
         <v>662</v>
       </c>
@@ -30338,7 +30338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="518" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="518" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A518" t="s">
         <v>722</v>
       </c>
@@ -30388,7 +30388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="519" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="519" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A519" t="s">
         <v>728</v>
       </c>
@@ -30438,7 +30438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="520" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="520" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A520" t="s">
         <v>840</v>
       </c>
@@ -30488,7 +30488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="521" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="521" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A521" t="s">
         <v>973</v>
       </c>
@@ -30588,7 +30588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="523" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="523" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A523" t="s">
         <v>32</v>
       </c>
@@ -30638,7 +30638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="524" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="524" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A524" t="s">
         <v>508</v>
       </c>
@@ -30688,7 +30688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="525" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="525" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A525" t="s">
         <v>508</v>
       </c>
@@ -30738,7 +30738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="526" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="526" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A526" t="s">
         <v>1032</v>
       </c>
@@ -30788,7 +30788,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="527" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="527" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A527" t="s">
         <v>141</v>
       </c>
@@ -30838,7 +30838,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="528" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="528" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A528" t="s">
         <v>187</v>
       </c>
@@ -30888,7 +30888,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="529" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="529" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A529" t="s">
         <v>353</v>
       </c>
@@ -30938,7 +30938,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="530" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="530" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A530" t="s">
         <v>366</v>
       </c>
@@ -31038,7 +31038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="532" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="532" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A532" t="s">
         <v>462</v>
       </c>
@@ -31188,7 +31188,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="535" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="535" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A535" t="s">
         <v>409</v>
       </c>
@@ -31238,7 +31238,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="536" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="536" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A536" t="s">
         <v>416</v>
       </c>
@@ -31288,7 +31288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="537" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="537" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A537" t="s">
         <v>476</v>
       </c>
@@ -31338,7 +31338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="538" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="538" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A538" t="s">
         <v>576</v>
       </c>
@@ -31438,7 +31438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="540" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="540" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A540" t="s">
         <v>263</v>
       </c>
@@ -31588,7 +31588,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="543" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="543" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A543" t="s">
         <v>541</v>
       </c>
@@ -31638,7 +31638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="544" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="544" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A544" t="s">
         <v>193</v>
       </c>
@@ -31688,7 +31688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="545" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="545" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A545" t="s">
         <v>193</v>
       </c>
@@ -31738,7 +31738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="546" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="546" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A546" t="s">
         <v>477</v>
       </c>
@@ -31788,7 +31788,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="547" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="547" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A547" t="s">
         <v>477</v>
       </c>
@@ -31838,7 +31838,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="548" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="548" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A548" t="s">
         <v>480</v>
       </c>
@@ -31888,7 +31888,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="549" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="549" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A549" t="s">
         <v>480</v>
       </c>
@@ -32538,7 +32538,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="562" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="562" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A562" t="s">
         <v>483</v>
       </c>
@@ -32588,7 +32588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="563" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="563" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A563" t="s">
         <v>483</v>
       </c>
@@ -32638,7 +32638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="564" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="564" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A564" t="s">
         <v>699</v>
       </c>
@@ -32688,7 +32688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="565" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="565" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A565" t="s">
         <v>701</v>
       </c>
@@ -32988,7 +32988,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="571" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="571" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A571" t="s">
         <v>998</v>
       </c>
@@ -33038,7 +33038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="572" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="572" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A572" t="s">
         <v>1000</v>
       </c>
@@ -33088,7 +33088,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="573" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="573" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A573" t="s">
         <v>1002</v>
       </c>
@@ -33138,7 +33138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="574" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="574" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A574" t="s">
         <v>1164</v>
       </c>
@@ -33288,7 +33288,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="577" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="577" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A577" t="s">
         <v>1166</v>
       </c>
@@ -33338,7 +33338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="578" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="578" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A578" t="s">
         <v>1168</v>
       </c>
@@ -33388,7 +33388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="579" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="579" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A579" t="s">
         <v>491</v>
       </c>
@@ -33438,7 +33438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="580" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="580" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A580" t="s">
         <v>494</v>
       </c>
@@ -33538,7 +33538,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="582" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="582" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A582" t="s">
         <v>710</v>
       </c>
@@ -33588,7 +33588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="583" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="583" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A583" t="s">
         <v>715</v>
       </c>
@@ -33638,7 +33638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="584" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="584" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A584" t="s">
         <v>997</v>
       </c>
@@ -33688,7 +33688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="585" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="585" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A585" t="s">
         <v>1004</v>
       </c>
@@ -33738,7 +33738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="586" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="586" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A586" t="s">
         <v>1006</v>
       </c>
@@ -33788,7 +33788,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="587" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="587" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A587" t="s">
         <v>1014</v>
       </c>
@@ -33838,7 +33838,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="588" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="588" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A588" t="s">
         <v>1016</v>
       </c>
@@ -33888,7 +33888,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="589" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="589" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A589" t="s">
         <v>1016</v>
       </c>
@@ -33938,7 +33938,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="590" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="590" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A590" t="s">
         <v>1016</v>
       </c>
@@ -33988,7 +33988,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="591" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="591" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A591" t="s">
         <v>1016</v>
       </c>
@@ -34038,7 +34038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="592" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="592" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A592" t="s">
         <v>1130</v>
       </c>
@@ -34088,7 +34088,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="593" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="593" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A593" t="s">
         <v>1176</v>
       </c>
@@ -34288,7 +34288,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="597" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="597" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A597" t="s">
         <v>1183</v>
       </c>
@@ -34688,7 +34688,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="605" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="605" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A605" t="s">
         <v>1189</v>
       </c>
@@ -34738,7 +34738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="606" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="606" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A606" t="s">
         <v>1191</v>
       </c>
@@ -34788,7 +34788,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="607" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="607" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A607" t="s">
         <v>1191</v>
       </c>
@@ -34838,7 +34838,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="608" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="608" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A608" t="s">
         <v>803</v>
       </c>
@@ -34938,7 +34938,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="610" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="610" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A610" t="s">
         <v>1010</v>
       </c>
@@ -34988,7 +34988,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="611" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="611" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A611" t="s">
         <v>1178</v>
       </c>
@@ -35038,7 +35038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="612" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="612" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A612" t="s">
         <v>492</v>
       </c>
@@ -35088,7 +35088,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="613" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="613" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A613" t="s">
         <v>711</v>
       </c>
@@ -35138,7 +35138,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="614" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="614" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A614" t="s">
         <v>713</v>
       </c>
@@ -35188,7 +35188,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="615" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="615" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A615" t="s">
         <v>1012</v>
       </c>
@@ -35238,7 +35238,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="616" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="616" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A616" t="s">
         <v>1170</v>
       </c>
@@ -35288,7 +35288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="617" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="617" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A617" t="s">
         <v>1170</v>
       </c>
@@ -35438,7 +35438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="620" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="620" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A620" t="s">
         <v>1180</v>
       </c>
@@ -35488,7 +35488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="621" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="621" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A621" t="s">
         <v>1180</v>
       </c>
@@ -35544,6 +35544,11 @@
       <customFilters>
         <customFilter operator="greaterThan" val="400"/>
       </customFilters>
+    </filterColumn>
+    <filterColumn colId="9">
+      <filters>
+        <filter val="TYPE_WATER"/>
+      </filters>
     </filterColumn>
     <filterColumn colId="15">
       <filters>

</xml_diff>

<commit_message>
Changed Route 1 and 6
</commit_message>
<xml_diff>
--- a/all_generations_pokemon_families.xlsx
+++ b/all_generations_pokemon_families.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\apetronack\Documents\Projects\pokefirered-expansion\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Austin\Documents\PokemonDecompBuild\pokefirered-expansion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{640D09F9-2BEB-4A1E-ABBB-ACCC28723074}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DC3E173-CD0D-4AE9-91D1-60A79C85DC6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{913F818F-7E2F-42B8-8FB9-B28A63806581}"/>
+    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{913F818F-7E2F-42B8-8FB9-B28A63806581}"/>
   </bookViews>
   <sheets>
     <sheet name="all_generations_pokemon_familie" sheetId="1" r:id="rId1"/>
@@ -4638,7 +4638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="4" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>929</v>
       </c>
@@ -4688,7 +4688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="5" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>929</v>
       </c>
@@ -6388,7 +6388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="39" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>759</v>
       </c>
@@ -7638,7 +7638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="64" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>197</v>
       </c>
@@ -8338,7 +8338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="78" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>369</v>
       </c>
@@ -8488,7 +8488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="81" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>581</v>
       </c>
@@ -8688,7 +8688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="85" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>775</v>
       </c>
@@ -9838,7 +9838,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="108" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>284</v>
       </c>
@@ -10188,7 +10188,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="115" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>913</v>
       </c>
@@ -10738,7 +10738,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="126" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>729</v>
       </c>
@@ -10988,7 +10988,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="131" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>34</v>
       </c>
@@ -11338,7 +11338,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="138" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>509</v>
       </c>
@@ -11388,7 +11388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="139" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>1033</v>
       </c>
@@ -11438,7 +11438,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="140" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>245</v>
       </c>
@@ -11488,7 +11488,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="141" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>245</v>
       </c>
@@ -11788,7 +11788,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="147" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>175</v>
       </c>
@@ -13688,7 +13688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="185" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
         <v>531</v>
       </c>
@@ -14038,7 +14038,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="192" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
         <v>1086</v>
       </c>
@@ -14238,7 +14238,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="196" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
         <v>226</v>
       </c>
@@ -14638,7 +14638,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="204" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A204" t="s">
         <v>380</v>
       </c>
@@ -14688,7 +14688,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="205" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A205" t="s">
         <v>762</v>
       </c>
@@ -15238,7 +15238,7 @@
         <v>1196</v>
       </c>
     </row>
-    <row r="216" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A216" t="s">
         <v>555</v>
       </c>
@@ -15288,7 +15288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="217" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A217" t="s">
         <v>674</v>
       </c>
@@ -15338,7 +15338,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="218" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A218" t="s">
         <v>974</v>
       </c>
@@ -15388,7 +15388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="219" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A219" t="s">
         <v>974</v>
       </c>
@@ -16388,7 +16388,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="239" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A239" t="s">
         <v>778</v>
       </c>
@@ -16538,7 +16538,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="242" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A242" t="s">
         <v>200</v>
       </c>
@@ -16588,7 +16588,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="243" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A243" t="s">
         <v>200</v>
       </c>
@@ -17288,7 +17288,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="257" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A257" t="s">
         <v>871</v>
       </c>
@@ -35540,11 +35540,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:P621" xr:uid="{6A7ECD2C-6F5B-4E4D-962E-4B55F2FEEDC6}">
-    <filterColumn colId="8">
-      <customFilters>
-        <customFilter operator="greaterThan" val="400"/>
-      </customFilters>
-    </filterColumn>
     <filterColumn colId="9">
       <filters>
         <filter val="TYPE_WATER"/>

</xml_diff>

<commit_message>
Updated growth rates for slow, fluctuating growth rate pokemon
</commit_message>
<xml_diff>
--- a/all_generations_pokemon_families.xlsx
+++ b/all_generations_pokemon_families.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\apetronack\Documents\Projects\pokefirered-expansion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D960E841-7FA1-44BA-950B-9B05A023D678}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{8F5A88A5-85B3-4260-B9DF-7B6D611872F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{CFD33D56-DCEE-4C8F-A281-92D9AA7B5F95}"/>
   </bookViews>
@@ -4301,7 +4301,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>41</v>
       </c>
@@ -4403,7 +4403,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>706</v>
       </c>
@@ -4439,7 +4439,7 @@
         <v>88</v>
       </c>
       <c r="L5" t="s">
-        <v>180</v>
+        <v>44</v>
       </c>
       <c r="M5" t="s">
         <v>708</v>
@@ -4454,7 +4454,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>847</v>
       </c>
@@ -4607,7 +4607,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>46</v>
       </c>
@@ -4811,7 +4811,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>522</v>
       </c>
@@ -4862,7 +4862,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>128</v>
       </c>
@@ -4913,7 +4913,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>473</v>
       </c>
@@ -5015,7 +5015,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>666</v>
       </c>
@@ -5066,7 +5066,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>670</v>
       </c>
@@ -5117,7 +5117,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>956</v>
       </c>
@@ -5168,7 +5168,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>962</v>
       </c>
@@ -5219,7 +5219,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>55</v>
       </c>
@@ -5576,7 +5576,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>592</v>
       </c>
@@ -5627,7 +5627,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>596</v>
       </c>
@@ -5663,7 +5663,7 @@
         <v>91</v>
       </c>
       <c r="L29" t="s">
-        <v>180</v>
+        <v>19</v>
       </c>
       <c r="M29" t="s">
         <v>598</v>
@@ -5729,7 +5729,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>698</v>
       </c>
@@ -5780,7 +5780,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>97</v>
       </c>
@@ -5831,7 +5831,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>104</v>
       </c>
@@ -5882,7 +5882,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>485</v>
       </c>
@@ -5933,7 +5933,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>686</v>
       </c>
@@ -5984,7 +5984,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>735</v>
       </c>
@@ -6086,7 +6086,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>996</v>
       </c>
@@ -6137,7 +6137,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>970</v>
       </c>
@@ -6341,7 +6341,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>709</v>
       </c>
@@ -6377,7 +6377,7 @@
         <v>88</v>
       </c>
       <c r="L43" t="s">
-        <v>180</v>
+        <v>44</v>
       </c>
       <c r="M43" t="s">
         <v>710</v>
@@ -6392,7 +6392,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>723</v>
       </c>
@@ -6494,7 +6494,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>169</v>
       </c>
@@ -6545,7 +6545,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>477</v>
       </c>
@@ -6596,7 +6596,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>552</v>
       </c>
@@ -6647,7 +6647,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>26</v>
       </c>
@@ -6698,7 +6698,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>79</v>
       </c>
@@ -6749,7 +6749,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>115</v>
       </c>
@@ -6800,7 +6800,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>208</v>
       </c>
@@ -6851,7 +6851,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>336</v>
       </c>
@@ -6902,7 +6902,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>93</v>
       </c>
@@ -7004,7 +7004,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>143</v>
       </c>
@@ -7106,7 +7106,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>186</v>
       </c>
@@ -7157,7 +7157,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>218</v>
       </c>
@@ -7208,7 +7208,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>218</v>
       </c>
@@ -7259,7 +7259,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>218</v>
       </c>
@@ -7310,7 +7310,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>218</v>
       </c>
@@ -7361,7 +7361,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>394</v>
       </c>
@@ -7412,7 +7412,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>444</v>
       </c>
@@ -7514,7 +7514,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>528</v>
       </c>
@@ -7565,7 +7565,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>528</v>
       </c>
@@ -7616,7 +7616,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>528</v>
       </c>
@@ -7667,7 +7667,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>528</v>
       </c>
@@ -7820,7 +7820,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>636</v>
       </c>
@@ -7871,7 +7871,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>670</v>
       </c>
@@ -7922,7 +7922,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>702</v>
       </c>
@@ -8009,7 +8009,7 @@
         <v>17</v>
       </c>
       <c r="L75" t="s">
-        <v>720</v>
+        <v>19</v>
       </c>
       <c r="M75" t="s">
         <v>721</v>
@@ -8024,7 +8024,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>729</v>
       </c>
@@ -8111,7 +8111,7 @@
         <v>171</v>
       </c>
       <c r="L77" t="s">
-        <v>720</v>
+        <v>19</v>
       </c>
       <c r="M77" t="s">
         <v>743</v>
@@ -8177,7 +8177,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>761</v>
       </c>
@@ -8228,7 +8228,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>765</v>
       </c>
@@ -8264,7 +8264,7 @@
         <v>81</v>
       </c>
       <c r="L80" t="s">
-        <v>180</v>
+        <v>19</v>
       </c>
       <c r="M80" t="s">
         <v>767</v>
@@ -8279,7 +8279,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>805</v>
       </c>
@@ -8381,7 +8381,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>835</v>
       </c>
@@ -8432,7 +8432,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>859</v>
       </c>
@@ -8483,7 +8483,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>863</v>
       </c>
@@ -8585,7 +8585,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>879</v>
       </c>
@@ -8636,7 +8636,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>885</v>
       </c>
@@ -8738,7 +8738,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>909</v>
       </c>
@@ -8789,7 +8789,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>1021</v>
       </c>
@@ -8840,7 +8840,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>1029</v>
       </c>
@@ -8891,7 +8891,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>1045</v>
       </c>
@@ -8978,7 +8978,7 @@
         <v>18</v>
       </c>
       <c r="L94" t="s">
-        <v>720</v>
+        <v>19</v>
       </c>
       <c r="M94" t="s">
         <v>783</v>
@@ -8993,7 +8993,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>265</v>
       </c>
@@ -9029,7 +9029,7 @@
         <v>36</v>
       </c>
       <c r="L95" t="s">
-        <v>180</v>
+        <v>731</v>
       </c>
       <c r="M95" t="s">
         <v>267</v>
@@ -9044,7 +9044,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>147</v>
       </c>
@@ -9197,7 +9197,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="99" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>202</v>
       </c>
@@ -9299,7 +9299,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="101" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>502</v>
       </c>
@@ -9401,7 +9401,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="103" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>793</v>
       </c>
@@ -9488,7 +9488,7 @@
         <v>36</v>
       </c>
       <c r="L104" t="s">
-        <v>720</v>
+        <v>19</v>
       </c>
       <c r="M104" t="s">
         <v>833</v>
@@ -9503,7 +9503,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="105" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>460</v>
       </c>
@@ -9554,7 +9554,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="106" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>944</v>
       </c>
@@ -9605,7 +9605,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="107" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>196</v>
       </c>
@@ -9656,7 +9656,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="108" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>269</v>
       </c>
@@ -9707,7 +9707,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="109" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>251</v>
       </c>
@@ -9758,7 +9758,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="110" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>648</v>
       </c>
@@ -9809,7 +9809,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="111" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>654</v>
       </c>
@@ -9860,7 +9860,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="112" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>660</v>
       </c>
@@ -9911,7 +9911,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="113" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>815</v>
       </c>
@@ -10013,7 +10013,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="115" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>34</v>
       </c>
@@ -10064,7 +10064,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="116" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>467</v>
       </c>
@@ -10115,7 +10115,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="117" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>950</v>
       </c>
@@ -10166,7 +10166,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="118" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>233</v>
       </c>
@@ -10217,7 +10217,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="119" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>233</v>
       </c>
@@ -10268,7 +10268,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="120" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>233</v>
       </c>
@@ -10319,7 +10319,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="121" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>233</v>
       </c>
@@ -10370,7 +10370,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="122" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>233</v>
       </c>
@@ -10421,7 +10421,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="123" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>233</v>
       </c>
@@ -10472,7 +10472,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="124" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>15</v>
       </c>
@@ -10523,7 +10523,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="125" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>454</v>
       </c>
@@ -10574,7 +10574,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="126" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>938</v>
       </c>
@@ -10676,7 +10676,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="128" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>165</v>
       </c>
@@ -10727,7 +10727,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="129" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>300</v>
       </c>
@@ -10778,7 +10778,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="130" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>343</v>
       </c>
@@ -10829,7 +10829,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="131" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>498</v>
       </c>
@@ -10880,7 +10880,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="132" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>110</v>
       </c>
@@ -10931,7 +10931,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="133" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>242</v>
       </c>
@@ -11084,7 +11084,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="136" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>294</v>
       </c>
@@ -11120,7 +11120,7 @@
         <v>88</v>
       </c>
       <c r="L136" t="s">
-        <v>180</v>
+        <v>731</v>
       </c>
       <c r="M136" t="s">
         <v>296</v>
@@ -11135,7 +11135,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="137" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>294</v>
       </c>
@@ -11171,7 +11171,7 @@
         <v>88</v>
       </c>
       <c r="L137" t="s">
-        <v>180</v>
+        <v>731</v>
       </c>
       <c r="M137" t="s">
         <v>297</v>
@@ -11186,7 +11186,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="138" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>396</v>
       </c>
@@ -11237,7 +11237,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="139" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>396</v>
       </c>
@@ -11288,7 +11288,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="140" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>396</v>
       </c>
@@ -11339,7 +11339,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="141" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>396</v>
       </c>
@@ -11390,7 +11390,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="142" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>396</v>
       </c>
@@ -11441,7 +11441,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="143" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>396</v>
       </c>
@@ -11492,7 +11492,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="144" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>396</v>
       </c>
@@ -11747,7 +11747,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="149" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>280</v>
       </c>
@@ -11798,7 +11798,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="150" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>1017</v>
       </c>
@@ -11849,7 +11849,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="151" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>288</v>
       </c>
@@ -11900,7 +11900,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="152" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>288</v>
       </c>
@@ -11951,7 +11951,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="153" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>288</v>
       </c>
@@ -12002,7 +12002,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="154" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>288</v>
       </c>
@@ -12053,7 +12053,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="155" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>489</v>
       </c>
@@ -12089,7 +12089,7 @@
         <v>81</v>
       </c>
       <c r="L155" t="s">
-        <v>180</v>
+        <v>19</v>
       </c>
       <c r="M155" t="s">
         <v>491</v>
@@ -12206,7 +12206,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="158" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>616</v>
       </c>
@@ -12242,7 +12242,7 @@
         <v>28</v>
       </c>
       <c r="L158" t="s">
-        <v>180</v>
+        <v>44</v>
       </c>
       <c r="M158" t="s">
         <v>618</v>
@@ -12257,7 +12257,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="159" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>620</v>
       </c>
@@ -12308,7 +12308,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="160" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>755</v>
       </c>
@@ -12344,7 +12344,7 @@
         <v>185</v>
       </c>
       <c r="L160" t="s">
-        <v>180</v>
+        <v>19</v>
       </c>
       <c r="M160" t="s">
         <v>757</v>
@@ -12359,7 +12359,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="161" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>799</v>
       </c>
@@ -12461,7 +12461,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="163" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
         <v>992</v>
       </c>
@@ -12512,7 +12512,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="164" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
         <v>1037</v>
       </c>
@@ -12548,7 +12548,7 @@
         <v>91</v>
       </c>
       <c r="L164" t="s">
-        <v>180</v>
+        <v>44</v>
       </c>
       <c r="M164" t="s">
         <v>1039</v>
@@ -12563,7 +12563,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="165" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>1041</v>
       </c>
@@ -12599,7 +12599,7 @@
         <v>43</v>
       </c>
       <c r="L165" t="s">
-        <v>180</v>
+        <v>112</v>
       </c>
       <c r="M165" t="s">
         <v>1043</v>
@@ -12665,7 +12665,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="167" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
         <v>1055</v>
       </c>
@@ -12701,7 +12701,7 @@
         <v>95</v>
       </c>
       <c r="L167" t="s">
-        <v>180</v>
+        <v>19</v>
       </c>
       <c r="M167" t="s">
         <v>1057</v>
@@ -12716,7 +12716,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="168" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
         <v>214</v>
       </c>
@@ -12752,7 +12752,7 @@
         <v>18</v>
       </c>
       <c r="L168" t="s">
-        <v>180</v>
+        <v>44</v>
       </c>
       <c r="M168" t="s">
         <v>216</v>
@@ -12767,7 +12767,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="169" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
         <v>811</v>
       </c>
@@ -12818,7 +12818,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="170" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
         <v>347</v>
       </c>
@@ -12854,7 +12854,7 @@
         <v>36</v>
       </c>
       <c r="L170" t="s">
-        <v>180</v>
+        <v>731</v>
       </c>
       <c r="M170" t="s">
         <v>349</v>
@@ -12869,7 +12869,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="171" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
         <v>313</v>
       </c>
@@ -12971,7 +12971,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="173" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>689</v>
       </c>
@@ -13073,7 +13073,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="175" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
         <v>808</v>
       </c>
@@ -13124,7 +13124,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="176" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
         <v>959</v>
       </c>
@@ -13175,7 +13175,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="177" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
         <v>318</v>
       </c>
@@ -13211,7 +13211,7 @@
         <v>185</v>
       </c>
       <c r="L177" t="s">
-        <v>180</v>
+        <v>731</v>
       </c>
       <c r="M177" t="s">
         <v>320</v>
@@ -13226,7 +13226,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="178" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
         <v>508</v>
       </c>
@@ -13277,7 +13277,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="179" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
         <v>891</v>
       </c>
@@ -13328,7 +13328,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="180" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
         <v>891</v>
       </c>
@@ -13415,7 +13415,7 @@
         <v>33</v>
       </c>
       <c r="L181" t="s">
-        <v>720</v>
+        <v>19</v>
       </c>
       <c r="M181" t="s">
         <v>1009</v>
@@ -13430,7 +13430,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="182" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
         <v>59</v>
       </c>
@@ -13481,7 +13481,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="183" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
         <v>178</v>
       </c>
@@ -13517,7 +13517,7 @@
         <v>28</v>
       </c>
       <c r="L183" t="s">
-        <v>180</v>
+        <v>731</v>
       </c>
       <c r="M183" t="s">
         <v>181</v>
@@ -13532,7 +13532,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="184" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
         <v>178</v>
       </c>
@@ -13568,7 +13568,7 @@
         <v>28</v>
       </c>
       <c r="L184" t="s">
-        <v>180</v>
+        <v>731</v>
       </c>
       <c r="M184" t="s">
         <v>182</v>
@@ -13583,7 +13583,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="185" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
         <v>178</v>
       </c>
@@ -13619,7 +13619,7 @@
         <v>185</v>
       </c>
       <c r="L185" t="s">
-        <v>180</v>
+        <v>731</v>
       </c>
       <c r="M185" t="s">
         <v>184</v>
@@ -13634,7 +13634,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="186" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
         <v>976</v>
       </c>
@@ -13685,7 +13685,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="187" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
         <v>980</v>
       </c>
@@ -13736,7 +13736,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="188" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
         <v>423</v>
       </c>
@@ -13787,7 +13787,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="189" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
         <v>427</v>
       </c>
@@ -13838,7 +13838,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="190" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
         <v>839</v>
       </c>
@@ -13889,7 +13889,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="191" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
         <v>843</v>
       </c>
@@ -13940,7 +13940,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="192" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
         <v>367</v>
       </c>
@@ -14042,7 +14042,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="194" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
         <v>733</v>
       </c>
@@ -14093,7 +14093,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="195" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
         <v>973</v>
       </c>
@@ -14144,7 +14144,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="196" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
         <v>100</v>
       </c>
@@ -14195,7 +14195,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="197" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
         <v>107</v>
       </c>
@@ -14246,7 +14246,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="198" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A198" t="s">
         <v>374</v>
       </c>
@@ -14297,7 +14297,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="199" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A199" t="s">
         <v>505</v>
       </c>
@@ -14348,7 +14348,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="200" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
         <v>738</v>
       </c>
@@ -14603,7 +14603,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="205" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A205" t="s">
         <v>48</v>
       </c>
@@ -14654,7 +14654,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="206" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A206" t="s">
         <v>275</v>
       </c>
@@ -14705,7 +14705,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="207" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A207" t="s">
         <v>189</v>
       </c>
@@ -14756,7 +14756,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="208" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A208" t="s">
         <v>189</v>
       </c>
@@ -14858,7 +14858,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="210" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A210" t="s">
         <v>211</v>
       </c>
@@ -14909,7 +14909,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="211" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A211" t="s">
         <v>222</v>
       </c>
@@ -14960,7 +14960,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="212" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A212" t="s">
         <v>222</v>
       </c>
@@ -15011,7 +15011,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="213" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A213" t="s">
         <v>222</v>
       </c>
@@ -15062,7 +15062,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="214" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A214" t="s">
         <v>222</v>
       </c>
@@ -15113,7 +15113,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="215" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A215" t="s">
         <v>415</v>
       </c>
@@ -15368,7 +15368,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="220" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
         <v>199</v>
       </c>
@@ -15419,7 +15419,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="221" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A221" t="s">
         <v>199</v>
       </c>
@@ -15470,7 +15470,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="222" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
         <v>777</v>
       </c>
@@ -15557,7 +15557,7 @@
         <v>36</v>
       </c>
       <c r="L223" t="s">
-        <v>720</v>
+        <v>19</v>
       </c>
       <c r="M223" t="s">
         <v>791</v>
@@ -15572,7 +15572,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="224" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A224" t="s">
         <v>30</v>
       </c>
@@ -15623,7 +15623,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="225" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
         <v>38</v>
       </c>
@@ -15674,7 +15674,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="226" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
         <v>205</v>
       </c>
@@ -15725,7 +15725,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="227" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
         <v>205</v>
       </c>
@@ -15776,7 +15776,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="228" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
         <v>272</v>
       </c>
@@ -15827,7 +15827,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="229" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
         <v>272</v>
       </c>
@@ -15878,7 +15878,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="230" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
         <v>22</v>
       </c>
@@ -15929,7 +15929,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="231" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
         <v>457</v>
       </c>
@@ -15980,7 +15980,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="232" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
         <v>463</v>
       </c>
@@ -16031,7 +16031,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="233" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
         <v>463</v>
       </c>
@@ -16082,7 +16082,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="234" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
         <v>470</v>
       </c>
@@ -16133,7 +16133,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="235" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
         <v>535</v>
       </c>
@@ -16235,7 +16235,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="237" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A237" t="s">
         <v>651</v>
       </c>
@@ -16286,7 +16286,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="238" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A238" t="s">
         <v>657</v>
       </c>
@@ -16337,7 +16337,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="239" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A239" t="s">
         <v>663</v>
       </c>
@@ -16490,7 +16490,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="242" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A242" t="s">
         <v>941</v>
       </c>
@@ -16541,7 +16541,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="243" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A243" t="s">
         <v>947</v>
       </c>
@@ -16592,7 +16592,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="244" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A244" t="s">
         <v>953</v>
       </c>
@@ -16949,7 +16949,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="251" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A251" t="s">
         <v>639</v>
       </c>
@@ -17000,7 +17000,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="252" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A252" t="s">
         <v>888</v>
       </c>
@@ -17051,7 +17051,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="253" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A253" t="s">
         <v>965</v>
       </c>
@@ -17102,7 +17102,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="254" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A254" t="s">
         <v>1032</v>
       </c>
@@ -17306,7 +17306,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="258" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A258" t="s">
         <v>447</v>
       </c>
@@ -17663,7 +17663,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="265" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A265" t="s">
         <v>912</v>
       </c>
@@ -17867,7 +17867,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="269" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A269" t="s">
         <v>476</v>
       </c>
@@ -17918,7 +17918,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="270" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A270" t="s">
         <v>493</v>
       </c>
@@ -18020,7 +18020,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="272" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A272" t="s">
         <v>753</v>
       </c>
@@ -18173,7 +18173,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="275" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A275" t="s">
         <v>559</v>
       </c>
@@ -18224,7 +18224,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="276" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A276" t="s">
         <v>576</v>
       </c>
@@ -18275,7 +18275,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="277" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
         <v>576</v>
       </c>
@@ -18326,7 +18326,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="278" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A278" t="s">
         <v>576</v>
       </c>
@@ -18377,7 +18377,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="279" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A279" t="s">
         <v>576</v>
       </c>
@@ -18428,7 +18428,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="280" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A280" t="s">
         <v>758</v>
       </c>
@@ -18464,7 +18464,7 @@
         <v>185</v>
       </c>
       <c r="L280" t="s">
-        <v>180</v>
+        <v>19</v>
       </c>
       <c r="M280" t="s">
         <v>759</v>
@@ -18530,7 +18530,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="282" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A282" t="s">
         <v>539</v>
       </c>
@@ -18581,7 +18581,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="283" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A283" t="s">
         <v>339</v>
       </c>
@@ -18683,7 +18683,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="285" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A285" t="s">
         <v>726</v>
       </c>
@@ -18887,7 +18887,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="289" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A289" t="s">
         <v>480</v>
       </c>
@@ -18938,7 +18938,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="290" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A290" t="s">
         <v>705</v>
       </c>
@@ -18989,7 +18989,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="291" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A291" t="s">
         <v>89</v>
       </c>
@@ -19040,7 +19040,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="292" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A292" t="s">
         <v>89</v>
       </c>
@@ -19091,7 +19091,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="293" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A293" t="s">
         <v>150</v>
       </c>
@@ -19244,7 +19244,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="296" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A296" t="s">
         <v>488</v>
       </c>
@@ -19346,7 +19346,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="298" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A298" t="s">
         <v>999</v>
       </c>
@@ -19397,7 +19397,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="299" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A299" t="s">
         <v>999</v>
       </c>
@@ -19703,7 +19703,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="305" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A305" t="s">
         <v>173</v>
       </c>
@@ -19958,7 +19958,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="310" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A310" t="s">
         <v>351</v>
       </c>
@@ -20009,7 +20009,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="311" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A311" t="s">
         <v>595</v>
       </c>
@@ -20162,7 +20162,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="314" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A314" t="s">
         <v>351</v>
       </c>
@@ -20213,7 +20213,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="315" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A315" t="s">
         <v>351</v>
       </c>
@@ -20264,7 +20264,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="316" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A316" t="s">
         <v>673</v>
       </c>
@@ -20315,7 +20315,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="317" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A317" t="s">
         <v>673</v>
       </c>
@@ -20366,7 +20366,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="318" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A318" t="s">
         <v>764</v>
       </c>
@@ -20417,7 +20417,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="319" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A319" t="s">
         <v>823</v>
       </c>
@@ -20468,7 +20468,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="320" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A320" t="s">
         <v>825</v>
       </c>
@@ -20519,7 +20519,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="321" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A321" t="s">
         <v>870</v>
       </c>
@@ -20555,7 +20555,7 @@
         <v>33</v>
       </c>
       <c r="L321" t="s">
-        <v>180</v>
+        <v>112</v>
       </c>
       <c r="M321" t="s">
         <v>25</v>
@@ -20723,7 +20723,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="325" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A325" t="s">
         <v>146</v>
       </c>
@@ -20774,7 +20774,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="326" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A326" t="s">
         <v>303</v>
       </c>
@@ -20825,7 +20825,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="327" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A327" t="s">
         <v>303</v>
       </c>
@@ -20876,7 +20876,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="328" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A328" t="s">
         <v>254</v>
       </c>
@@ -20978,7 +20978,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="330" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A330" t="s">
         <v>669</v>
       </c>
@@ -21029,7 +21029,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="331" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A331" t="s">
         <v>802</v>
       </c>
@@ -21080,7 +21080,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="332" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A332" t="s">
         <v>114</v>
       </c>
@@ -21182,7 +21182,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="334" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A334" t="s">
         <v>532</v>
       </c>
@@ -21233,7 +21233,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="335" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A335" t="s">
         <v>534</v>
       </c>
@@ -21284,7 +21284,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="336" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A336" t="s">
         <v>547</v>
       </c>
@@ -21335,7 +21335,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="337" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A337" t="s">
         <v>701</v>
       </c>
@@ -21437,7 +21437,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="339" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A339" t="s">
         <v>768</v>
       </c>
@@ -21473,7 +21473,7 @@
         <v>81</v>
       </c>
       <c r="L339" t="s">
-        <v>180</v>
+        <v>19</v>
       </c>
       <c r="M339" t="s">
         <v>25</v>
@@ -21539,7 +21539,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="341" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A341" t="s">
         <v>797</v>
       </c>
@@ -21590,7 +21590,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="342" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A342" t="s">
         <v>862</v>
       </c>
@@ -21641,7 +21641,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="343" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A343" t="s">
         <v>866</v>
       </c>
@@ -21794,7 +21794,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="346" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A346" t="s">
         <v>61</v>
       </c>
@@ -21845,7 +21845,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="347" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A347" t="s">
         <v>1020</v>
       </c>
@@ -21896,7 +21896,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="348" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A348" t="s">
         <v>292</v>
       </c>
@@ -21947,7 +21947,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="349" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A349" t="s">
         <v>292</v>
       </c>
@@ -22049,7 +22049,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="351" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A351" t="s">
         <v>492</v>
       </c>
@@ -22085,7 +22085,7 @@
         <v>81</v>
       </c>
       <c r="L351" t="s">
-        <v>180</v>
+        <v>19</v>
       </c>
       <c r="M351" t="s">
         <v>25</v>
@@ -22100,7 +22100,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="352" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A352" t="s">
         <v>614</v>
       </c>
@@ -22136,7 +22136,7 @@
         <v>33</v>
       </c>
       <c r="L352" t="s">
-        <v>180</v>
+        <v>731</v>
       </c>
       <c r="M352" t="s">
         <v>25</v>
@@ -22238,7 +22238,7 @@
         <v>67</v>
       </c>
       <c r="L354" t="s">
-        <v>720</v>
+        <v>19</v>
       </c>
       <c r="M354" t="s">
         <v>25</v>
@@ -22253,7 +22253,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="355" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A355" t="s">
         <v>1011</v>
       </c>
@@ -22304,7 +22304,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="356" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A356" t="s">
         <v>1087</v>
       </c>
@@ -22442,7 +22442,7 @@
         <v>171</v>
       </c>
       <c r="L358" t="s">
-        <v>720</v>
+        <v>19</v>
       </c>
       <c r="M358" t="s">
         <v>25</v>
@@ -22508,7 +22508,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="360" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A360" t="s">
         <v>321</v>
       </c>
@@ -22544,7 +22544,7 @@
         <v>185</v>
       </c>
       <c r="L360" t="s">
-        <v>180</v>
+        <v>731</v>
       </c>
       <c r="M360" t="s">
         <v>322</v>
@@ -22559,7 +22559,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="361" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A361" t="s">
         <v>796</v>
       </c>
@@ -22610,7 +22610,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="362" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A362" t="s">
         <v>814</v>
       </c>
@@ -22763,7 +22763,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="365" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A365" t="s">
         <v>961</v>
       </c>
@@ -22814,7 +22814,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="366" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A366" t="s">
         <v>1027</v>
       </c>
@@ -22865,7 +22865,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="367" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A367" t="s">
         <v>370</v>
       </c>
@@ -22916,7 +22916,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="368" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A368" t="s">
         <v>201</v>
       </c>
@@ -22967,7 +22967,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="369" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A369" t="s">
         <v>334</v>
       </c>
@@ -23018,7 +23018,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="370" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A370" t="s">
         <v>316</v>
       </c>
@@ -23324,7 +23324,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="376" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A376" t="s">
         <v>511</v>
       </c>
@@ -23426,7 +23426,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="378" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A378" t="s">
         <v>628</v>
       </c>
@@ -23513,7 +23513,7 @@
         <v>171</v>
       </c>
       <c r="L379" t="s">
-        <v>720</v>
+        <v>19</v>
       </c>
       <c r="M379" t="s">
         <v>25</v>
@@ -23528,7 +23528,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="380" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A380" t="s">
         <v>377</v>
       </c>
@@ -23579,7 +23579,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="381" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A381" t="s">
         <v>426</v>
       </c>
@@ -23630,7 +23630,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="382" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="382" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A382" t="s">
         <v>430</v>
       </c>
@@ -23681,7 +23681,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="383" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="383" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A383" t="s">
         <v>283</v>
       </c>
@@ -23732,7 +23732,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="384" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="384" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A384" t="s">
         <v>542</v>
       </c>
@@ -23819,7 +23819,7 @@
         <v>18</v>
       </c>
       <c r="L385" t="s">
-        <v>720</v>
+        <v>19</v>
       </c>
       <c r="M385" t="s">
         <v>25</v>
@@ -23834,7 +23834,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="386" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="386" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A386" t="s">
         <v>842</v>
       </c>
@@ -23885,7 +23885,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="387" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="387" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A387" t="s">
         <v>846</v>
       </c>
@@ -23936,7 +23936,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="388" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="388" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A388" t="s">
         <v>979</v>
       </c>
@@ -23987,7 +23987,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="389" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="389" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A389" t="s">
         <v>983</v>
       </c>
@@ -24038,7 +24038,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="390" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="390" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A390" t="s">
         <v>995</v>
       </c>
@@ -24125,7 +24125,7 @@
         <v>33</v>
       </c>
       <c r="L391" t="s">
-        <v>720</v>
+        <v>19</v>
       </c>
       <c r="M391" t="s">
         <v>25</v>
@@ -24242,7 +24242,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="394" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="394" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A394" t="s">
         <v>168</v>
       </c>
@@ -24293,7 +24293,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="395" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="395" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A395" t="s">
         <v>612</v>
       </c>
@@ -24329,7 +24329,7 @@
         <v>33</v>
       </c>
       <c r="L395" t="s">
-        <v>180</v>
+        <v>731</v>
       </c>
       <c r="M395" t="s">
         <v>25</v>
@@ -24344,7 +24344,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="396" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="396" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A396" t="s">
         <v>85</v>
       </c>
@@ -24395,7 +24395,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="397" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="397" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A397" t="s">
         <v>356</v>
       </c>
@@ -24446,7 +24446,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="398" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="398" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A398" t="s">
         <v>356</v>
       </c>
@@ -24497,7 +24497,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="399" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="399" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A399" t="s">
         <v>274</v>
       </c>
@@ -24548,7 +24548,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="400" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="400" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A400" t="s">
         <v>381</v>
       </c>
@@ -24584,7 +24584,7 @@
         <v>43</v>
       </c>
       <c r="L400" t="s">
-        <v>180</v>
+        <v>731</v>
       </c>
       <c r="M400" t="s">
         <v>25</v>
@@ -24596,10 +24596,10 @@
         <v>0</v>
       </c>
       <c r="P400" t="s">
-        <v>1098</v>
-      </c>
-    </row>
-    <row r="401" spans="1:16" x14ac:dyDescent="0.35">
+        <v>1097</v>
+      </c>
+    </row>
+    <row r="401" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A401" t="s">
         <v>85</v>
       </c>
@@ -24803,7 +24803,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="405" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="405" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A405" t="s">
         <v>361</v>
       </c>
@@ -24854,7 +24854,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="406" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="406" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A406" t="s">
         <v>362</v>
       </c>
@@ -24905,7 +24905,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="407" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="407" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A407" t="s">
         <v>501</v>
       </c>
@@ -25007,7 +25007,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="409" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="409" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A409" t="s">
         <v>555</v>
       </c>
@@ -25058,7 +25058,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="410" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="410" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A410" t="s">
         <v>574</v>
       </c>
@@ -25094,7 +25094,7 @@
         <v>171</v>
       </c>
       <c r="L410" t="s">
-        <v>180</v>
+        <v>731</v>
       </c>
       <c r="M410" t="s">
         <v>25</v>
@@ -25211,7 +25211,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="413" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="413" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A413" t="s">
         <v>619</v>
       </c>
@@ -25247,7 +25247,7 @@
         <v>28</v>
       </c>
       <c r="L413" t="s">
-        <v>180</v>
+        <v>44</v>
       </c>
       <c r="M413" t="s">
         <v>25</v>
@@ -25262,7 +25262,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="414" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="414" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A414" t="s">
         <v>623</v>
       </c>
@@ -25313,7 +25313,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="415" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="415" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A415" t="s">
         <v>691</v>
       </c>
@@ -25451,7 +25451,7 @@
         <v>36</v>
       </c>
       <c r="L417" t="s">
-        <v>720</v>
+        <v>19</v>
       </c>
       <c r="M417" t="s">
         <v>25</v>
@@ -25466,7 +25466,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="418" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="418" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A418" t="s">
         <v>838</v>
       </c>
@@ -25517,7 +25517,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="419" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="419" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A419" t="s">
         <v>1024</v>
       </c>
@@ -25568,7 +25568,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="420" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="420" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A420" t="s">
         <v>1044</v>
       </c>
@@ -25604,7 +25604,7 @@
         <v>67</v>
       </c>
       <c r="L420" t="s">
-        <v>180</v>
+        <v>112</v>
       </c>
       <c r="M420" t="s">
         <v>25</v>
@@ -25619,7 +25619,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="421" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="421" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A421" t="s">
         <v>1048</v>
       </c>
@@ -25670,7 +25670,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="422" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="422" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A422" t="s">
         <v>1058</v>
       </c>
@@ -25706,7 +25706,7 @@
         <v>95</v>
       </c>
       <c r="L422" t="s">
-        <v>180</v>
+        <v>19</v>
       </c>
       <c r="M422" t="s">
         <v>25</v>
@@ -25721,7 +25721,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="423" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="423" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A423" t="s">
         <v>103</v>
       </c>
@@ -25772,7 +25772,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="424" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="424" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A424" t="s">
         <v>109</v>
       </c>
@@ -25823,7 +25823,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="425" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="425" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A425" t="s">
         <v>119</v>
       </c>
@@ -25925,7 +25925,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="427" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="427" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A427" t="s">
         <v>572</v>
       </c>
@@ -25976,7 +25976,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="428" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="428" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A428" t="s">
         <v>780</v>
       </c>
@@ -26078,7 +26078,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="430" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="430" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A430" t="s">
         <v>194</v>
       </c>
@@ -26180,7 +26180,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="432" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="432" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A432" t="s">
         <v>195</v>
       </c>
@@ -26231,7 +26231,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="433" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="433" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A433" t="s">
         <v>225</v>
       </c>
@@ -26282,7 +26282,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="434" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="434" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A434" t="s">
         <v>225</v>
       </c>
@@ -26333,7 +26333,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="435" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="435" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A435" t="s">
         <v>238</v>
       </c>
@@ -26384,7 +26384,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="436" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="436" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A436" t="s">
         <v>240</v>
       </c>
@@ -26435,7 +26435,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="437" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="437" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A437" t="s">
         <v>238</v>
       </c>
@@ -26486,7 +26486,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="438" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="438" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A438" t="s">
         <v>240</v>
       </c>
@@ -26537,7 +26537,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="439" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="439" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A439" t="s">
         <v>279</v>
       </c>
@@ -26639,7 +26639,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="441" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="441" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A441" t="s">
         <v>581</v>
       </c>
@@ -26690,7 +26690,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="442" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="442" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A442" t="s">
         <v>583</v>
       </c>
@@ -26792,7 +26792,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="444" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="444" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A444" t="s">
         <v>818</v>
       </c>
@@ -26843,7 +26843,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="445" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="445" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A445" t="s">
         <v>882</v>
       </c>
@@ -26894,7 +26894,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="446" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="446" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A446" t="s">
         <v>883</v>
       </c>
@@ -26945,7 +26945,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="447" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="447" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A447" t="s">
         <v>897</v>
       </c>
@@ -26996,7 +26996,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="448" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="448" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A448" t="s">
         <v>898</v>
       </c>
@@ -27047,7 +27047,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="449" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="449" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A449" t="s">
         <v>217</v>
       </c>
@@ -27098,7 +27098,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="450" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="450" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A450" t="s">
         <v>431</v>
       </c>
@@ -27134,7 +27134,7 @@
         <v>33</v>
       </c>
       <c r="L450" t="s">
-        <v>180</v>
+        <v>19</v>
       </c>
       <c r="M450" t="s">
         <v>25</v>
@@ -27200,7 +27200,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="452" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="452" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A452" t="s">
         <v>419</v>
       </c>
@@ -27302,7 +27302,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="454" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="454" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A454" t="s">
         <v>538</v>
       </c>
@@ -27353,7 +27353,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="455" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="455" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A455" t="s">
         <v>711</v>
       </c>
@@ -27389,7 +27389,7 @@
         <v>88</v>
       </c>
       <c r="L455" t="s">
-        <v>180</v>
+        <v>44</v>
       </c>
       <c r="M455" t="s">
         <v>25</v>
@@ -27404,7 +27404,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="456" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="456" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A456" t="s">
         <v>712</v>
       </c>
@@ -27440,7 +27440,7 @@
         <v>171</v>
       </c>
       <c r="L456" t="s">
-        <v>180</v>
+        <v>44</v>
       </c>
       <c r="M456" t="s">
         <v>25</v>
@@ -27455,7 +27455,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="457" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="457" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A457" t="s">
         <v>350</v>
       </c>
@@ -27491,7 +27491,7 @@
         <v>88</v>
       </c>
       <c r="L457" t="s">
-        <v>180</v>
+        <v>731</v>
       </c>
       <c r="M457" t="s">
         <v>25</v>
@@ -27506,7 +27506,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="458" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="458" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A458" t="s">
         <v>213</v>
       </c>
@@ -27557,7 +27557,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="459" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="459" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A459" t="s">
         <v>298</v>
       </c>
@@ -27593,7 +27593,7 @@
         <v>88</v>
       </c>
       <c r="L459" t="s">
-        <v>180</v>
+        <v>731</v>
       </c>
       <c r="M459" t="s">
         <v>297</v>
@@ -27608,7 +27608,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="460" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="460" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A460" t="s">
         <v>298</v>
       </c>
@@ -27644,7 +27644,7 @@
         <v>299</v>
       </c>
       <c r="L460" t="s">
-        <v>180</v>
+        <v>731</v>
       </c>
       <c r="M460" t="s">
         <v>296</v>
@@ -27659,7 +27659,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="461" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="461" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A461" t="s">
         <v>355</v>
       </c>
@@ -27710,7 +27710,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="462" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="462" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A462" t="s">
         <v>507</v>
       </c>
@@ -27761,7 +27761,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="463" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="463" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A463" t="s">
         <v>551</v>
       </c>
@@ -27914,7 +27914,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="466" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="466" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A466" t="s">
         <v>677</v>
       </c>
@@ -27965,7 +27965,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="467" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="467" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A467" t="s">
         <v>740</v>
       </c>
@@ -28016,7 +28016,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="468" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="468" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A468" t="s">
         <v>810</v>
       </c>
@@ -28322,7 +28322,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="474" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="474" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A474" t="s">
         <v>975</v>
       </c>
@@ -28373,7 +28373,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="475" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="475" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A475" t="s">
         <v>406</v>
       </c>
@@ -28424,7 +28424,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="476" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="476" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A476" t="s">
         <v>407</v>
       </c>
@@ -28475,7 +28475,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="477" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="477" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A477" t="s">
         <v>408</v>
       </c>
@@ -28526,7 +28526,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="478" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="478" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A478" t="s">
         <v>268</v>
       </c>
@@ -28562,7 +28562,7 @@
         <v>95</v>
       </c>
       <c r="L478" t="s">
-        <v>180</v>
+        <v>731</v>
       </c>
       <c r="M478" t="s">
         <v>25</v>
@@ -28577,7 +28577,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="479" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="479" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A479" t="s">
         <v>24</v>
       </c>
@@ -28628,7 +28628,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="480" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="480" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A480" t="s">
         <v>207</v>
       </c>
@@ -28679,7 +28679,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="481" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="481" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A481" t="s">
         <v>409</v>
       </c>
@@ -28730,7 +28730,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="482" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="482" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A482" t="s">
         <v>410</v>
       </c>
@@ -28781,7 +28781,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="483" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="483" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A483" t="s">
         <v>411</v>
       </c>
@@ -28832,7 +28832,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="484" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="484" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A484" t="s">
         <v>412</v>
       </c>
@@ -28934,7 +28934,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="486" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="486" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A486" t="s">
         <v>459</v>
       </c>
@@ -28985,7 +28985,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="487" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="487" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A487" t="s">
         <v>563</v>
       </c>
@@ -29138,7 +29138,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="490" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="490" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A490" t="s">
         <v>869</v>
       </c>
@@ -29189,7 +29189,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="491" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="491" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A491" t="s">
         <v>943</v>
       </c>
@@ -29240,7 +29240,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="492" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="492" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A492" t="s">
         <v>1035</v>
       </c>
@@ -29291,7 +29291,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="493" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="493" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A493" t="s">
         <v>1040</v>
       </c>
@@ -29327,7 +29327,7 @@
         <v>91</v>
       </c>
       <c r="L493" t="s">
-        <v>180</v>
+        <v>44</v>
       </c>
       <c r="M493" t="s">
         <v>25</v>
@@ -29342,7 +29342,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="494" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="494" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A494" t="s">
         <v>40</v>
       </c>
@@ -29393,7 +29393,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="495" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="495" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A495" t="s">
         <v>472</v>
       </c>
@@ -29444,7 +29444,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="496" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="496" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A496" t="s">
         <v>599</v>
       </c>
@@ -29480,7 +29480,7 @@
         <v>91</v>
       </c>
       <c r="L496" t="s">
-        <v>180</v>
+        <v>44</v>
       </c>
       <c r="M496" t="s">
         <v>25</v>
@@ -29495,7 +29495,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="497" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="497" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A497" t="s">
         <v>653</v>
       </c>
@@ -29546,7 +29546,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="498" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="498" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A498" t="s">
         <v>659</v>
       </c>
@@ -29597,7 +29597,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="499" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="499" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A499" t="s">
         <v>760</v>
       </c>
@@ -29633,7 +29633,7 @@
         <v>185</v>
       </c>
       <c r="L499" t="s">
-        <v>180</v>
+        <v>19</v>
       </c>
       <c r="M499" t="s">
         <v>25</v>
@@ -29648,7 +29648,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="500" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="500" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A500" t="s">
         <v>890</v>
       </c>
@@ -29699,7 +29699,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="501" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="501" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A501" t="s">
         <v>955</v>
       </c>
@@ -29750,7 +29750,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="502" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="502" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A502" t="s">
         <v>32</v>
       </c>
@@ -29801,7 +29801,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="503" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="503" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A503" t="s">
         <v>466</v>
       </c>
@@ -29852,7 +29852,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="504" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="504" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A504" t="s">
         <v>466</v>
       </c>
@@ -29903,7 +29903,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="505" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="505" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A505" t="s">
         <v>949</v>
       </c>
@@ -29954,7 +29954,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="506" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="506" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A506" t="s">
         <v>392</v>
       </c>
@@ -29990,7 +29990,7 @@
         <v>95</v>
       </c>
       <c r="L506" t="s">
-        <v>180</v>
+        <v>19</v>
       </c>
       <c r="M506" t="s">
         <v>25</v>
@@ -30005,7 +30005,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="507" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="507" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A507" t="s">
         <v>131</v>
       </c>
@@ -30056,7 +30056,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="508" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="508" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A508" t="s">
         <v>176</v>
       </c>
@@ -30107,7 +30107,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="509" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="509" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A509" t="s">
         <v>324</v>
       </c>
@@ -30143,7 +30143,7 @@
         <v>185</v>
       </c>
       <c r="L509" t="s">
-        <v>180</v>
+        <v>731</v>
       </c>
       <c r="M509" t="s">
         <v>25</v>
@@ -30158,7 +30158,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="510" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="510" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A510" t="s">
         <v>332</v>
       </c>
@@ -30209,7 +30209,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="511" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="511" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A511" t="s">
         <v>422</v>
       </c>
@@ -30260,7 +30260,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="512" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="512" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A512" t="s">
         <v>665</v>
       </c>
@@ -30311,7 +30311,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="513" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="513" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A513" t="s">
         <v>433</v>
       </c>
@@ -30464,7 +30464,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="516" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="516" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A516" t="s">
         <v>342</v>
       </c>
@@ -30515,7 +30515,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="517" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="517" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A517" t="s">
         <v>373</v>
       </c>
@@ -30566,7 +30566,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="518" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="518" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A518" t="s">
         <v>380</v>
       </c>
@@ -30617,7 +30617,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="519" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="519" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A519" t="s">
         <v>525</v>
       </c>
@@ -30668,7 +30668,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="520" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="520" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A520" t="s">
         <v>851</v>
       </c>
@@ -30719,7 +30719,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="521" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="521" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A521" t="s">
         <v>245</v>
       </c>
@@ -30770,7 +30770,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="522" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="522" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A522" t="s">
         <v>497</v>
       </c>
@@ -30872,7 +30872,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="524" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="524" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A524" t="s">
         <v>183</v>
       </c>
@@ -30908,7 +30908,7 @@
         <v>28</v>
       </c>
       <c r="L524" t="s">
-        <v>180</v>
+        <v>731</v>
       </c>
       <c r="M524" t="s">
         <v>184</v>
@@ -30923,7 +30923,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="525" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="525" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A525" t="s">
         <v>183</v>
       </c>
@@ -30959,7 +30959,7 @@
         <v>185</v>
       </c>
       <c r="L525" t="s">
-        <v>180</v>
+        <v>731</v>
       </c>
       <c r="M525" t="s">
         <v>181</v>
@@ -31025,7 +31025,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="527" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="527" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A527" t="s">
         <v>435</v>
       </c>
@@ -31076,7 +31076,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="528" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="528" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A528" t="s">
         <v>438</v>
       </c>
@@ -31127,7 +31127,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="529" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="529" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A529" t="s">
         <v>441</v>
       </c>
@@ -31178,7 +31178,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="530" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="530" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A530" t="s">
         <v>435</v>
       </c>
@@ -31229,7 +31229,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="531" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="531" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A531" t="s">
         <v>438</v>
       </c>
@@ -31280,7 +31280,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="532" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="532" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A532" t="s">
         <v>441</v>
       </c>
@@ -31331,7 +31331,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="533" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="533" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A533" t="s">
         <v>630</v>
       </c>
@@ -31382,7 +31382,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="534" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="534" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A534" t="s">
         <v>632</v>
       </c>
@@ -31433,7 +31433,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="535" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="535" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A535" t="s">
         <v>634</v>
       </c>
@@ -31484,7 +31484,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="536" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="536" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A536" t="s">
         <v>915</v>
       </c>
@@ -31535,7 +31535,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="537" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="537" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A537" t="s">
         <v>917</v>
       </c>
@@ -31586,7 +31586,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="538" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="538" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A538" t="s">
         <v>919</v>
       </c>
@@ -31637,7 +31637,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="539" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="539" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A539" t="s">
         <v>1066</v>
       </c>
@@ -31688,7 +31688,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="540" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="540" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A540" t="s">
         <v>1068</v>
       </c>
@@ -31739,7 +31739,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="541" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="541" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A541" t="s">
         <v>1070</v>
       </c>
@@ -31790,7 +31790,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="542" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="542" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A542" t="s">
         <v>449</v>
       </c>
@@ -31841,7 +31841,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="543" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="543" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A543" t="s">
         <v>452</v>
       </c>
@@ -31892,7 +31892,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="544" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="544" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A544" t="s">
         <v>641</v>
       </c>
@@ -31943,7 +31943,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="545" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="545" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A545" t="s">
         <v>646</v>
       </c>
@@ -32045,7 +32045,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="547" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="547" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A547" t="s">
         <v>914</v>
       </c>
@@ -32096,7 +32096,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="548" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="548" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A548" t="s">
         <v>921</v>
       </c>
@@ -32147,7 +32147,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="549" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="549" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A549" t="s">
         <v>923</v>
       </c>
@@ -32198,7 +32198,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="550" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="550" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A550" t="s">
         <v>931</v>
       </c>
@@ -32249,7 +32249,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="551" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="551" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A551" t="s">
         <v>933</v>
       </c>
@@ -32300,7 +32300,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="552" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="552" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A552" t="s">
         <v>933</v>
       </c>
@@ -32351,7 +32351,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="553" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="553" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A553" t="s">
         <v>933</v>
       </c>
@@ -32402,7 +32402,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="554" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="554" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A554" t="s">
         <v>933</v>
       </c>
@@ -32453,7 +32453,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="555" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="555" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A555" t="s">
         <v>1034</v>
       </c>
@@ -32504,7 +32504,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="556" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="556" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A556" t="s">
         <v>1078</v>
       </c>
@@ -32555,7 +32555,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="557" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="557" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A557" t="s">
         <v>1085</v>
       </c>
@@ -32606,7 +32606,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="558" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="558" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A558" t="s">
         <v>1089</v>
       </c>
@@ -32657,7 +32657,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="559" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="559" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A559" t="s">
         <v>1091</v>
       </c>
@@ -32708,7 +32708,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="560" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="560" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A560" t="s">
         <v>1093</v>
       </c>
@@ -32759,7 +32759,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="561" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="561" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A561" t="s">
         <v>1093</v>
       </c>
@@ -32810,7 +32810,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="562" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="562" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A562" t="s">
         <v>728</v>
       </c>
@@ -32861,7 +32861,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="563" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="563" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A563" t="s">
         <v>925</v>
       </c>
@@ -32912,7 +32912,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="564" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="564" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A564" t="s">
         <v>927</v>
       </c>
@@ -32963,7 +32963,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="565" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="565" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A565" t="s">
         <v>1080</v>
       </c>
@@ -33014,7 +33014,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="566" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="566" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A566" t="s">
         <v>450</v>
       </c>
@@ -33065,7 +33065,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="567" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="567" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A567" t="s">
         <v>642</v>
       </c>
@@ -33116,7 +33116,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="568" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="568" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A568" t="s">
         <v>644</v>
       </c>
@@ -33167,7 +33167,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="569" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="569" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A569" t="s">
         <v>929</v>
       </c>
@@ -33218,7 +33218,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="570" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="570" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A570" t="s">
         <v>1072</v>
       </c>
@@ -33320,7 +33320,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="572" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="572" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A572" t="s">
         <v>1075</v>
       </c>
@@ -33422,7 +33422,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="574" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="574" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A574" t="s">
         <v>1082</v>
       </c>
@@ -33526,6 +33526,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:P575" xr:uid="{DA2BF836-2FD5-4520-BC72-6D688307FCF3}">
+    <filterColumn colId="11">
+      <filters>
+        <filter val="GROWTH_FLUCTUATING"/>
+      </filters>
+    </filterColumn>
     <filterColumn colId="15">
       <filters>
         <filter val="Y"/>
@@ -33536,5 +33541,6 @@
     <sortCondition ref="I1:I575"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>